<commit_message>
Ronda 12/10 11:55: respuestas de WhatsApp, Marketplace, tienda nueva del Supermall; oficina con estado real de cada agente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H75" headerRowCount="1">
-  <autoFilter ref="A1:H75"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H76" headerRowCount="1">
+  <autoFilter ref="A1:H76"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -1269,7 +1269,9 @@
       <c r="G12" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="H12" s="2" t="n"/>
+      <c r="H12" s="8" t="n">
+        <v>2150</v>
+      </c>
       <c r="I12" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -2264,7 +2266,9 @@
         <v>59.99</v>
       </c>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
+      <c r="G9" s="8" t="n">
+        <v>2150</v>
+      </c>
       <c r="H9" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A9,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A9,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -3471,7 +3475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6333,6 +6337,44 @@
         </is>
       </c>
       <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Compucenter (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="n">
+        <v>2150</v>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (Corsair Vengeance RGB DDR4 16GB 3600; no dice si es 2x8; Bs 2.560 con factura)</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -6414,10 +6456,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId75"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId76"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Informe diario 12/10 con precios reales de eBay, reportes regenerados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSYxqiVsX36QqKNYdTUdvM
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Historial" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Ronda 12/10 12:10: respuestas de Supermall y PC Components, Corsair DDR5 5600 en Marketplace, reportes y oficina
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Historial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H76" headerRowCount="1">
-  <autoFilter ref="A1:H76"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H82" headerRowCount="1">
+  <autoFilter ref="A1:H82"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -982,12 +982,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>SSD NVMe 1TB</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -996,20 +996,18 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>329</v>
+        <v>114.99</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>283.99</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>4800</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>5664</v>
-      </c>
+        <v>1800</v>
+      </c>
+      <c r="H8" s="2" t="n"/>
       <c r="I8" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1019,7 +1017,7 @@
         <v/>
       </c>
       <c r="K8" s="8" t="n">
-        <v>350</v>
+        <v>80</v>
       </c>
       <c r="L8" s="11">
         <f>IF(D8="","",MIN(MAX(Supuestos!$B$5,CEILING((K8*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D8*Supuestos!$B$9))</f>
@@ -1049,12 +1047,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1063,18 +1061,20 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>114.99</v>
+        <v>329</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>99.98999999999999</v>
+        <v>283.99</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="H9" s="2" t="n"/>
+        <v>4800</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>4760</v>
+      </c>
       <c r="I9" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1084,7 +1084,7 @@
         <v/>
       </c>
       <c r="K9" s="8" t="n">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="L9" s="11">
         <f>IF(D9="","",MIN(MAX(Supuestos!$B$5,CEILING((K9*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D9*Supuestos!$B$9))</f>
@@ -1311,12 +1311,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-13400</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>RAM</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1325,18 +1325,18 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>259.78</v>
+        <v>485</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>149.99</v>
-      </c>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="8" t="n">
-        <v>2300</v>
-      </c>
+        <v>399.99</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H13" s="2" t="n"/>
       <c r="I13" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1346,7 +1346,7 @@
         <v/>
       </c>
       <c r="K13" s="8" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="L13" s="11">
         <f>IF(D13="","",MIN(MAX(Supuestos!$B$5,CEILING((K13*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D13*Supuestos!$B$9))</f>
@@ -1376,7 +1376,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 5600</t>
+          <t>Intel Core i5-13400</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1390,16 +1390,18 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>138.9</v>
+        <v>259.78</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>135</v>
+        <v>149.99</v>
       </c>
       <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
+      <c r="H14" s="8" t="n">
+        <v>2300</v>
+      </c>
       <c r="I14" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1409,7 +1411,7 @@
         <v/>
       </c>
       <c r="K14" s="8" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="L14" s="11">
         <f>IF(D14="","",MIN(MAX(Supuestos!$B$5,CEILING((K14*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D14*Supuestos!$B$9))</f>
@@ -1439,7 +1441,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 5700X3D</t>
+          <t>Ryzen 5 5600</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -1452,10 +1454,14 @@
           <t>ver en eBay</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
+      <c r="D15" s="7" t="n">
+        <v>138.9</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="F15" s="7" t="n">
-        <v>305</v>
+        <v>135</v>
       </c>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
@@ -1498,7 +1504,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>Ryzen 7 5700X3D</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1511,14 +1517,10 @@
           <t>ver en eBay</t>
         </is>
       </c>
-      <c r="D16" s="7" t="n">
-        <v>144.25</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
       <c r="F16" s="7" t="n">
-        <v>122.99</v>
+        <v>305</v>
       </c>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
@@ -1561,7 +1563,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-12400F</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1575,13 +1577,13 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>150</v>
+        <v>144.25</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>119.95</v>
+        <v>122.99</v>
       </c>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
@@ -1594,7 +1596,7 @@
         <v/>
       </c>
       <c r="K17" s="8" t="n">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="L17" s="11">
         <f>IF(D17="","",MIN(MAX(Supuestos!$B$5,CEILING((K17*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D17*Supuestos!$B$9))</f>
@@ -1624,12 +1626,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+          <t>Intel Core i5-12400F</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>RAM</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -1638,13 +1640,13 @@
         </is>
       </c>
       <c r="D18" s="7" t="n">
-        <v>485</v>
+        <v>150</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>399.99</v>
+        <v>119.95</v>
       </c>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
@@ -1657,7 +1659,7 @@
         <v/>
       </c>
       <c r="K18" s="8" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="L18" s="11">
         <f>IF(D18="","",MIN(MAX(Supuestos!$B$5,CEILING((K18*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D18*Supuestos!$B$9))</f>
@@ -1995,7 +1997,9 @@
         <v>454.99</v>
       </c>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="8" t="n">
+        <v>6140</v>
+      </c>
       <c r="H4" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A4,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A4,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2051,7 +2055,7 @@
       </c>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="8" t="n">
-        <v>5664</v>
+        <v>4760</v>
       </c>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
@@ -2597,7 +2601,9 @@
       <c r="E15" s="7" t="n">
         <v>399.99</v>
       </c>
-      <c r="F15" s="2" t="n"/>
+      <c r="F15" s="8" t="n">
+        <v>4500</v>
+      </c>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A15,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A15,Dólar!$A:$A,0))),"")</f>
@@ -3475,7 +3481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6375,6 +6381,234 @@
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 9 9950X</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Tienda Supermall (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="n">
+        <v>6140</v>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (garantía 6 meses)</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Tienda Supermall (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="n">
+        <v>4760</v>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (la tienda lo ofrece como "7700x3d"; foto de caja 7800X3D; stock bajo; garantía 6 meses; confirmar modelo)</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="n">
+        <v>6800</v>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>no indicado</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (Kingston NV3 PCIe 4.0; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="E81" s="11" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (marca "ediloca" PCIe 4.0; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E82" s="11" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>usado como nuevo (4 meses de uso; publicado hace 7 semanas)</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -6457,10 +6691,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId81"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId76"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId82"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda 12/10 16:35 (PC de la casa): respuestas de PC Components, Supermall y Electro-TTS; comparación, reportes y oficina
- PC Components (SCZ): Corsair DDR5 32GB 6000 Bs 6.700 c/u llevando 2 (referencia).
- Supermall: 9950X a precio final, sin descuento por cantidad.
- Electro-TTS respondió "No case" (dudoso).
- Fila de PC Components en tiendas-cochabamba.csv corregida (tenía comas sin comillas).
- comparar.py --tc 11.90, reportes.py y oficina/generar.py; oficina republicada. Sin chats nuevos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H82" headerRowCount="1">
-  <autoFilter ref="A1:H82"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H83" headerRowCount="1">
+  <autoFilter ref="A1:H83"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -3481,7 +3481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6609,6 +6609,44 @@
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="E83" s="11" t="n">
+        <v>6700</v>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (precio c/u llevando 2; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -6697,10 +6735,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId82"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId83"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catálogo de Punto Tecnológico (tienda del Supermall) y columna tienda vs Marketplace en la oficina
- 16 precios de puntotecnologic.com: 10 cuentan (14400F, 265K, 7600, 12400F, DDR4 Corsair 2x8, SSD 1TB y 2TB) y 6 no (agotados con precios viejos u otra marca).
- Primeros precios locales del Ryzen 5 7600 (Bs 2.860) y el i5-12400F (Bs 2.460).
- Oficina: columna "Tienda vs Mkt" (precio estándar contra mercado informal) y fila de resumen al pie.
- comparar.py --tc 11.90, reportes.py y oficina/generar.py; oficina republicada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H83" headerRowCount="1">
-  <autoFilter ref="A1:H83"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H99" headerRowCount="1">
+  <autoFilter ref="A1:H99"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -785,12 +785,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 2TB</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -799,18 +799,18 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>209.99</v>
+        <v>144.25</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>179.99</v>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>3550</v>
-      </c>
-      <c r="H5" s="2" t="n"/>
+        <v>122.99</v>
+      </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="8" t="n">
+        <v>2860</v>
+      </c>
       <c r="I5" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -820,7 +820,7 @@
         <v/>
       </c>
       <c r="K5" s="8" t="n">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="L5" s="11">
         <f>IF(D5="","",MIN(MAX(Supuestos!$B$5,CEILING((K5*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D5*Supuestos!$B$9))</f>
@@ -850,12 +850,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Intel Core Ultra 7 265K</t>
+          <t>SSD NVMe 2TB</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -864,17 +864,19 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>244.87</v>
+        <v>209.99</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>209.99</v>
-      </c>
-      <c r="G6" s="2" t="n"/>
+        <v>179.99</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>3550</v>
+      </c>
       <c r="H6" s="8" t="n">
-        <v>3950</v>
+        <v>4060</v>
       </c>
       <c r="I6" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -885,7 +887,7 @@
         <v/>
       </c>
       <c r="K6" s="8" t="n">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="L6" s="11">
         <f>IF(D6="","",MIN(MAX(Supuestos!$B$5,CEILING((K6*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D6*Supuestos!$B$9))</f>
@@ -915,7 +917,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-14400F</t>
+          <t>Intel Core Ultra 7 265K</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -929,19 +931,17 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>164.49</v>
+        <v>244.87</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>136.99</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>2700</v>
-      </c>
+        <v>209.99</v>
+      </c>
+      <c r="G7" s="2" t="n"/>
       <c r="H7" s="8" t="n">
-        <v>2537</v>
+        <v>3950</v>
       </c>
       <c r="I7" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -952,7 +952,7 @@
         <v/>
       </c>
       <c r="K7" s="8" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="L7" s="11">
         <f>IF(D7="","",MIN(MAX(Supuestos!$B$5,CEILING((K7*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D7*Supuestos!$B$9))</f>
@@ -982,12 +982,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Intel Core i5-12400F</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -996,18 +996,18 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>114.99</v>
+        <v>150</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>99.98999999999999</v>
-      </c>
-      <c r="G8" s="8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="H8" s="2" t="n"/>
+        <v>119.95</v>
+      </c>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="8" t="n">
+        <v>2460</v>
+      </c>
       <c r="I8" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1017,7 +1017,7 @@
         <v/>
       </c>
       <c r="K8" s="8" t="n">
-        <v>80</v>
+        <v>250</v>
       </c>
       <c r="L8" s="11">
         <f>IF(D8="","",MIN(MAX(Supuestos!$B$5,CEILING((K8*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D8*Supuestos!$B$9))</f>
@@ -1047,7 +1047,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core i5-14400F</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1061,19 +1061,19 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>329</v>
+        <v>164.49</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>283.99</v>
+        <v>136.99</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>4800</v>
+        <v>2700</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>4760</v>
+        <v>2520</v>
       </c>
       <c r="I9" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1084,7 +1084,7 @@
         <v/>
       </c>
       <c r="K9" s="8" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="L9" s="11">
         <f>IF(D9="","",MIN(MAX(Supuestos!$B$5,CEILING((K9*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D9*Supuestos!$B$9))</f>
@@ -1114,12 +1114,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+          <t>SSD NVMe 1TB</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>RAM</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1128,18 +1128,20 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>425</v>
+        <v>114.99</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>10.99</v>
+        <v>0</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>399.9</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>6200</v>
-      </c>
-      <c r="H10" s="2" t="n"/>
+        <v>1800</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>1860</v>
+      </c>
       <c r="I10" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1149,7 +1151,7 @@
         <v/>
       </c>
       <c r="K10" s="8" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="L10" s="11">
         <f>IF(D10="","",MIN(MAX(Supuestos!$B$5,CEILING((K10*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D10*Supuestos!$B$9))</f>
@@ -1179,7 +1181,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 9 9950X</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1193,17 +1195,19 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>499.99</v>
+        <v>329</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>454.99</v>
-      </c>
-      <c r="G11" s="2" t="n"/>
+        <v>283.99</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>4800</v>
+      </c>
       <c r="H11" s="8" t="n">
-        <v>5580</v>
+        <v>4760</v>
       </c>
       <c r="I11" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1244,7 +1248,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR4 16GB (2x8) 3200</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1258,20 +1262,18 @@
         </is>
       </c>
       <c r="D12" s="7" t="n">
-        <v>75</v>
+        <v>425</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>0</v>
+        <v>10.99</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>59.99</v>
+        <v>399.9</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>2150</v>
-      </c>
+        <v>6200</v>
+      </c>
+      <c r="H12" s="2" t="n"/>
       <c r="I12" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1281,7 +1283,7 @@
         <v/>
       </c>
       <c r="K12" s="8" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="L12" s="11">
         <f>IF(D12="","",MIN(MAX(Supuestos!$B$5,CEILING((K12*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D12*Supuestos!$B$9))</f>
@@ -1311,12 +1313,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+          <t>Ryzen 9 9950X</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>RAM</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1325,18 +1327,18 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>485</v>
+        <v>499.99</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>399.99</v>
-      </c>
-      <c r="G13" s="8" t="n">
-        <v>4500</v>
-      </c>
-      <c r="H13" s="2" t="n"/>
+        <v>454.99</v>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="8" t="n">
+        <v>5580</v>
+      </c>
       <c r="I13" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1346,7 +1348,7 @@
         <v/>
       </c>
       <c r="K13" s="8" t="n">
-        <v>150</v>
+        <v>350</v>
       </c>
       <c r="L13" s="11">
         <f>IF(D13="","",MIN(MAX(Supuestos!$B$5,CEILING((K13*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D13*Supuestos!$B$9))</f>
@@ -1376,12 +1378,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-13400</t>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>RAM</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1390,17 +1392,19 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>259.78</v>
+        <v>75</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>149.99</v>
-      </c>
-      <c r="G14" s="2" t="n"/>
+        <v>59.99</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>900</v>
+      </c>
       <c r="H14" s="8" t="n">
-        <v>2300</v>
+        <v>2150</v>
       </c>
       <c r="I14" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1411,7 +1415,7 @@
         <v/>
       </c>
       <c r="K14" s="8" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="L14" s="11">
         <f>IF(D14="","",MIN(MAX(Supuestos!$B$5,CEILING((K14*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D14*Supuestos!$B$9))</f>
@@ -1441,12 +1445,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 5600</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>RAM</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1455,15 +1459,17 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>138.9</v>
+        <v>485</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>135</v>
-      </c>
-      <c r="G15" s="2" t="n"/>
+        <v>399.99</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>4500</v>
+      </c>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1474,7 +1480,7 @@
         <v/>
       </c>
       <c r="K15" s="8" t="n">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="L15" s="11">
         <f>IF(D15="","",MIN(MAX(Supuestos!$B$5,CEILING((K15*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D15*Supuestos!$B$9))</f>
@@ -1504,7 +1510,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 5700X3D</t>
+          <t>Intel Core i5-13400</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1517,13 +1523,19 @@
           <t>ver en eBay</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
+      <c r="D16" s="7" t="n">
+        <v>259.78</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="F16" s="7" t="n">
-        <v>305</v>
+        <v>149.99</v>
       </c>
       <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
+      <c r="H16" s="8" t="n">
+        <v>2300</v>
+      </c>
       <c r="I16" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1533,7 +1545,7 @@
         <v/>
       </c>
       <c r="K16" s="8" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="L16" s="11">
         <f>IF(D16="","",MIN(MAX(Supuestos!$B$5,CEILING((K16*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D16*Supuestos!$B$9))</f>
@@ -1563,7 +1575,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>Ryzen 5 5600</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1577,13 +1589,13 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>144.25</v>
+        <v>138.9</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>122.99</v>
+        <v>135</v>
       </c>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
@@ -1626,7 +1638,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-12400F</t>
+          <t>Ryzen 7 5700X3D</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1639,14 +1651,10 @@
           <t>ver en eBay</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n">
-        <v>150</v>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
       <c r="F18" s="7" t="n">
-        <v>119.95</v>
+        <v>305</v>
       </c>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
@@ -1659,7 +1667,7 @@
         <v/>
       </c>
       <c r="K18" s="8" t="n">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="L18" s="11">
         <f>IF(D18="","",MIN(MAX(Supuestos!$B$5,CEILING((K18*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D18*Supuestos!$B$9))</f>
@@ -1887,7 +1895,9 @@
         <v>179.99</v>
       </c>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="8" t="n">
+        <v>4060</v>
+      </c>
       <c r="H2" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A2,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A2,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -1942,7 +1952,9 @@
         <v>99.98999999999999</v>
       </c>
       <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="8" t="n">
+        <v>1860</v>
+      </c>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2162,7 +2174,9 @@
         <v>122.99</v>
       </c>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="8" t="n">
+        <v>2860</v>
+      </c>
       <c r="H7" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A7,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A7,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2328,7 +2342,7 @@
       </c>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="8" t="n">
-        <v>2537</v>
+        <v>2520</v>
       </c>
       <c r="H10" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))),"")</f>
@@ -2439,7 +2453,9 @@
         <v>119.95</v>
       </c>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="8" t="n">
+        <v>2460</v>
+      </c>
       <c r="H12" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A12,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A12,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2492,7 +2508,9 @@
         <v>209.99</v>
       </c>
       <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
+      <c r="G13" s="8" t="n">
+        <v>4290</v>
+      </c>
       <c r="H13" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A13,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A13,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -3481,7 +3499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6647,6 +6665,614 @@
         </is>
       </c>
       <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E84" s="11" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web)</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E85" s="11" t="n">
+        <v>4290</v>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>stock bajo (web; por WhatsApp dijeron que el 265K solo está en Santa Cruz)</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E86" s="11" t="n">
+        <v>2860</v>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>stock bajo (web)</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-12400F</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E87" s="11" t="n">
+        <v>2460</v>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web)</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E88" s="11" t="n">
+        <v>5360</v>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>agotado (web, "Ryzen 7 7800x3d Chip"; precio de referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 5600</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E89" s="11" t="n">
+        <v>1710</v>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>agotado (web; precio de referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-13400</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="n">
+        <v>2310</v>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>agotado (web; precio de referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E91" s="11" t="n">
+        <v>2160</v>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Corsair Vengeance RGB Pro TUF Gaming 2x8 3200)</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E92" s="11" t="n">
+        <v>5360</v>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>agotado (web; precio de referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E93" s="11" t="n">
+        <v>5660</v>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Patriot Viper 32GB 6000 RGB: otra marca; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E94" s="11" t="n">
+        <v>5860</v>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Kingston Fury 32GB 2x16 5200/5600: otra marca; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E95" s="11" t="n">
+        <v>1860</v>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>stock bajo (web; Hiksemi Wave M.2 1TB)</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E96" s="11" t="n">
+        <v>2060</v>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; WD SN3000 M.2 1TB)</t>
+        </is>
+      </c>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E97" s="11" t="n">
+        <v>2152</v>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Kingston NV3 M.2 1TB)</t>
+        </is>
+      </c>
+      <c r="H97" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 2TB</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E98" s="11" t="n">
+        <v>4060</v>
+      </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>stock bajo (web; Apacer M.2 2TB 7400 MB/s)</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 2TB</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E99" s="11" t="n">
+        <v>4560</v>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Hiksemi Futurex M.2 2TB)</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -6736,10 +7362,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId98"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId83"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId99"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda 12/10 17:40 (PC de la casa, en vivo): precios de Viadata y aduana en CLAUDE.md
- Viadata: 7800X3D OEM Bs 5.500; 5600X OEM Bs 2.500 y 265KF en caja Bs 5.200 como referencia (no cuentan).
- TecnoGamer solo mensaje automático; Display Importadora, T&T, Smart Cube y Geek Store sin respuesta.
- CLAUDE.md: la aduana suele ir incluida en el courier; se suma aparte cuando no.
- comparar.py --tc 11.90, reportes.py y generar.py; oficina republicada. Ronda seguida en vivo en vivo/_ronda.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H99" headerRowCount="1">
-  <autoFilter ref="A1:H99"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H102" headerRowCount="1">
+  <autoFilter ref="A1:H102"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -3499,7 +3499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7273,6 +7273,120 @@
         </is>
       </c>
       <c r="H99" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Viadata Computadoras (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E100" s="11" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (solo el chip)</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 5600</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>Viadata Computadoras (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E101" s="11" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (es el 5600X, no el 5600; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H101" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Viadata Computadoras (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E102" s="11" t="n">
+        <v>5200</v>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>nuevo en caja (es el 265KF, sin gráficos integrados; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -7378,10 +7492,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId101"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId99"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId102"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda 12/10 18:00 (Marketplace por Messenger): i5 14400 confirmado y SanDisk 2TB externo
- Mensajes por Messenger (cuenta del usuario, aprobados) al 7800X3D "sellado", al i5 14400 y a la Corsair DDR5 6000 RS.
- i5 14400: es el de gráficos (no el 14400F), nuevo en blíster, final Bs 2.700 → no cuenta; chat archivado.
- "SSD SanDisk 2TB" Bs 3.550: es externo portátil, no NVMe → no cuenta; el SSD 2TB pasa a 34 % contra Punto Tecnológico.
- El anuncio Bs 1 del 7800X3D es de Punto Tecnológico (ya cotizado): no se escribió.
- Captura del agente de Marketplace; comparación, reportes y oficina republicada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -785,12 +785,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>SSD NVMe 2TB</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -799,17 +799,17 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>144.25</v>
+        <v>209.99</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>122.99</v>
+        <v>179.99</v>
       </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="8" t="n">
-        <v>2860</v>
+        <v>4060</v>
       </c>
       <c r="I5" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -820,7 +820,7 @@
         <v/>
       </c>
       <c r="K5" s="8" t="n">
-        <v>350</v>
+        <v>80</v>
       </c>
       <c r="L5" s="11">
         <f>IF(D5="","",MIN(MAX(Supuestos!$B$5,CEILING((K5*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D5*Supuestos!$B$9))</f>
@@ -850,12 +850,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 2TB</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -864,19 +864,17 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>209.99</v>
+        <v>144.25</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>179.99</v>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>3550</v>
-      </c>
+        <v>122.99</v>
+      </c>
+      <c r="G6" s="2" t="n"/>
       <c r="H6" s="8" t="n">
-        <v>4060</v>
+        <v>2860</v>
       </c>
       <c r="I6" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -887,7 +885,7 @@
         <v/>
       </c>
       <c r="K6" s="8" t="n">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="L6" s="11">
         <f>IF(D6="","",MIN(MAX(Supuestos!$B$5,CEILING((K6*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D6*Supuestos!$B$9))</f>
@@ -1069,9 +1067,7 @@
       <c r="F9" s="7" t="n">
         <v>136.99</v>
       </c>
-      <c r="G9" s="8" t="n">
-        <v>2700</v>
-      </c>
+      <c r="G9" s="2" t="n"/>
       <c r="H9" s="8" t="n">
         <v>2520</v>
       </c>
@@ -2670,9 +2666,7 @@
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
-      <c r="F16" s="8" t="n">
-        <v>3550</v>
-      </c>
+      <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A16,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A16,Dólar!$A:$A,0))),"")</f>
@@ -2682,11 +2676,7 @@
         <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A16,Dólar!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>ver anuncio</t>
-        </is>
-      </c>
+      <c r="J16" s="2" t="n"/>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="16">
         <f>IF(OR($K16="",D16=""),"",IF(COUNTIFS($B:$B,$B16,$A:$A,$K16,D:D,"&gt;=0")=0,"",D16-SUMIFS(D:D,$B:$B,$B16,$A:$A,$K16)))</f>
@@ -2970,9 +2960,7 @@
       </c>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
-      <c r="F22" s="8" t="n">
-        <v>2700</v>
-      </c>
+      <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A22,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A22,Dólar!$A:$A,0))),"")</f>
@@ -2982,11 +2970,7 @@
         <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A22,Dólar!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>ver anuncio</t>
-        </is>
-      </c>
+      <c r="J22" s="2" t="n"/>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="16">
         <f>IF(OR($K22="",D22=""),"",IF(COUNTIFS($B:$B,$B22,$A:$A,$K22,D:D,"&gt;=0")=0,"",D22-SUMIFS(D:D,$B:$B,$B22,$A:$A,$K22)))</f>
@@ -3190,19 +3174,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5901,7 +5883,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>no indicado (anuncio dice i5 14400; confirmar si es F)</t>
+          <t>confirmado por Messenger el 12/10: es el i5-14400 con gráficos (no el F), nuevo en blíster, precio final Bs 2.700; no cuenta</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr">
@@ -6243,7 +6225,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>no indicado (SanDisk 2TB; no dice si es NVMe o SATA)</t>
+          <t>revisado el 12/10: es un SSD externo portátil SanDisk 2TB (1050 MB/s, USB con cable, IP65), no un NVMe interno; no cuenta</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Revisión diaria 2026-10-13: dólar, eBay, comparación e informe
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CJzLuJo8jFDB3Cz7QtEYZE
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -279,8 +279,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Historial" displayName="Historial" ref="A1:O25" headerRowCount="1">
-  <autoFilter ref="A1:O25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Historial" displayName="Historial" ref="A1:O39" headerRowCount="1">
+  <autoFilter ref="A1:O39"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Producto"/>
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H102" headerRowCount="1">
-  <autoFilter ref="A1:H102"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H128" headerRowCount="1">
+  <autoFilter ref="A1:H128"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -633,7 +633,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>¿Qué conviene traer? · 12/10/2026</t>
+          <t>¿Qué conviene traer? · 13/10/2026</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -785,12 +785,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 2TB</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -799,17 +799,17 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>209.99</v>
+        <v>143.24</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>179.99</v>
+        <v>122.99</v>
       </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="8" t="n">
-        <v>4060</v>
+        <v>2860</v>
       </c>
       <c r="I5" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -820,7 +820,7 @@
         <v/>
       </c>
       <c r="K5" s="8" t="n">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="L5" s="11">
         <f>IF(D5="","",MIN(MAX(Supuestos!$B$5,CEILING((K5*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D5*Supuestos!$B$9))</f>
@@ -850,12 +850,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>SSD NVMe 2TB</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -864,17 +864,17 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>144.25</v>
+        <v>209.99</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>122.99</v>
+        <v>170</v>
       </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="8" t="n">
-        <v>2860</v>
+        <v>4060</v>
       </c>
       <c r="I6" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -885,7 +885,7 @@
         <v/>
       </c>
       <c r="K6" s="8" t="n">
-        <v>350</v>
+        <v>80</v>
       </c>
       <c r="L6" s="11">
         <f>IF(D6="","",MIN(MAX(Supuestos!$B$5,CEILING((K6*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D6*Supuestos!$B$9))</f>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>244.87</v>
+        <v>234.99</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
@@ -1000,7 +1000,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>119.95</v>
+        <v>99</v>
       </c>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="8" t="n">
@@ -1065,7 +1065,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>136.99</v>
+        <v>134</v>
       </c>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="8" t="n">
@@ -1374,7 +1374,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR4 16GB (2x8) 3200</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1388,20 +1388,18 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>75</v>
+        <v>485</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>59.99</v>
+        <v>383.99</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>2150</v>
-      </c>
+        <v>4500</v>
+      </c>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1411,7 +1409,7 @@
         <v/>
       </c>
       <c r="K14" s="8" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="L14" s="11">
         <f>IF(D14="","",MIN(MAX(Supuestos!$B$5,CEILING((K14*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D14*Supuestos!$B$9))</f>
@@ -1441,7 +1439,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -1455,18 +1453,20 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>485</v>
+        <v>92.98999999999999</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>399.99</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>4500</v>
-      </c>
-      <c r="H15" s="2" t="n"/>
+        <v>900</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>2150</v>
+      </c>
       <c r="I15" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1476,7 +1476,7 @@
         <v/>
       </c>
       <c r="K15" s="8" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="L15" s="11">
         <f>IF(D15="","",MIN(MAX(Supuestos!$B$5,CEILING((K15*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D15*Supuestos!$B$9))</f>
@@ -1650,7 +1650,7 @@
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="7" t="n">
-        <v>305</v>
+        <v>299.99</v>
       </c>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
@@ -1773,7 +1773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1872,7 +1872,7 @@
     </row>
     <row r="2">
       <c r="A2" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
@@ -1888,12 +1888,10 @@
         <v>209.99</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>179.99</v>
+        <v>170</v>
       </c>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" s="8" t="n">
-        <v>4060</v>
-      </c>
+      <c r="G2" s="2" t="n"/>
       <c r="H2" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A2,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A2,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -1908,7 +1906,7 @@
         </is>
       </c>
       <c r="K2" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L2" s="16">
         <f>IF(OR($K2="",D2=""),"",IF(COUNTIFS($B:$B,$B2,$A:$A,$K2,D:D,"&gt;=0")=0,"",D2-SUMIFS(D:D,$B:$B,$B2,$A:$A,$K2)))</f>
@@ -1929,7 +1927,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
@@ -1948,9 +1946,7 @@
         <v>99.98999999999999</v>
       </c>
       <c r="F3" s="2" t="n"/>
-      <c r="G3" s="8" t="n">
-        <v>1860</v>
-      </c>
+      <c r="G3" s="2" t="n"/>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -1965,7 +1961,7 @@
         </is>
       </c>
       <c r="K3" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L3" s="16">
         <f>IF(OR($K3="",D3=""),"",IF(COUNTIFS($B:$B,$B3,$A:$A,$K3,D:D,"&gt;=0")=0,"",D3-SUMIFS(D:D,$B:$B,$B3,$A:$A,$K3)))</f>
@@ -1986,7 +1982,7 @@
     </row>
     <row r="4">
       <c r="A4" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
@@ -2005,9 +2001,7 @@
         <v>454.99</v>
       </c>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" s="8" t="n">
-        <v>6140</v>
-      </c>
+      <c r="G4" s="2" t="n"/>
       <c r="H4" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A4,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A4,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2022,7 +2016,7 @@
         </is>
       </c>
       <c r="K4" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L4" s="16">
         <f>IF(OR($K4="",D4=""),"",IF(COUNTIFS($B:$B,$B4,$A:$A,$K4,D:D,"&gt;=0")=0,"",D4-SUMIFS(D:D,$B:$B,$B4,$A:$A,$K4)))</f>
@@ -2043,7 +2037,7 @@
     </row>
     <row r="5">
       <c r="A5" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
@@ -2062,9 +2056,7 @@
         <v>283.99</v>
       </c>
       <c r="F5" s="2" t="n"/>
-      <c r="G5" s="8" t="n">
-        <v>4760</v>
-      </c>
+      <c r="G5" s="2" t="n"/>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2079,7 +2071,7 @@
         </is>
       </c>
       <c r="K5" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L5" s="16">
         <f>IF(OR($K5="",D5=""),"",IF(COUNTIFS($B:$B,$B5,$A:$A,$K5,D:D,"&gt;=0")=0,"",D5-SUMIFS(D:D,$B:$B,$B5,$A:$A,$K5)))</f>
@@ -2100,7 +2092,7 @@
     </row>
     <row r="6">
       <c r="A6" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
@@ -2114,7 +2106,7 @@
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="7" t="n">
-        <v>305</v>
+        <v>299.99</v>
       </c>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
@@ -2131,7 +2123,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K6" s="5" t="n"/>
+      <c r="K6" s="15" t="n">
+        <v>46307</v>
+      </c>
       <c r="L6" s="16">
         <f>IF(OR($K6="",D6=""),"",IF(COUNTIFS($B:$B,$B6,$A:$A,$K6,D:D,"&gt;=0")=0,"",D6-SUMIFS(D:D,$B:$B,$B6,$A:$A,$K6)))</f>
         <v/>
@@ -2151,7 +2145,7 @@
     </row>
     <row r="7">
       <c r="A7" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
@@ -2164,15 +2158,13 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>144.25</v>
+        <v>143.24</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>122.99</v>
       </c>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="8" t="n">
-        <v>2860</v>
-      </c>
+      <c r="G7" s="2" t="n"/>
       <c r="H7" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A7,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A7,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2187,7 +2179,7 @@
         </is>
       </c>
       <c r="K7" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L7" s="16">
         <f>IF(OR($K7="",D7=""),"",IF(COUNTIFS($B:$B,$B7,$A:$A,$K7,D:D,"&gt;=0")=0,"",D7-SUMIFS(D:D,$B:$B,$B7,$A:$A,$K7)))</f>
@@ -2208,7 +2200,7 @@
     </row>
     <row r="8">
       <c r="A8" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
@@ -2241,7 +2233,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K8" s="5" t="n"/>
+      <c r="K8" s="15" t="n">
+        <v>46307</v>
+      </c>
       <c r="L8" s="16">
         <f>IF(OR($K8="",D8=""),"",IF(COUNTIFS($B:$B,$B8,$A:$A,$K8,D:D,"&gt;=0")=0,"",D8-SUMIFS(D:D,$B:$B,$B8,$A:$A,$K8)))</f>
         <v/>
@@ -2261,7 +2255,7 @@
     </row>
     <row r="9">
       <c r="A9" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -2274,15 +2268,13 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>75</v>
+        <v>92.98999999999999</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>59.99</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="8" t="n">
-        <v>2150</v>
-      </c>
+      <c r="G9" s="2" t="n"/>
       <c r="H9" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A9,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A9,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2297,7 +2289,7 @@
         </is>
       </c>
       <c r="K9" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L9" s="16">
         <f>IF(OR($K9="",D9=""),"",IF(COUNTIFS($B:$B,$B9,$A:$A,$K9,D:D,"&gt;=0")=0,"",D9-SUMIFS(D:D,$B:$B,$B9,$A:$A,$K9)))</f>
@@ -2318,7 +2310,7 @@
     </row>
     <row r="10">
       <c r="A10" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
@@ -2334,12 +2326,10 @@
         <v>164.49</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>136.99</v>
+        <v>134</v>
       </c>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="8" t="n">
-        <v>2520</v>
-      </c>
+      <c r="G10" s="2" t="n"/>
       <c r="H10" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2354,7 +2344,7 @@
         </is>
       </c>
       <c r="K10" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L10" s="16">
         <f>IF(OR($K10="",D10=""),"",IF(COUNTIFS($B:$B,$B10,$A:$A,$K10,D:D,"&gt;=0")=0,"",D10-SUMIFS(D:D,$B:$B,$B10,$A:$A,$K10)))</f>
@@ -2375,7 +2365,7 @@
     </row>
     <row r="11">
       <c r="A11" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
@@ -2387,9 +2377,7 @@
           <t>CPU</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
-        <v>259.78</v>
-      </c>
+      <c r="D11" s="2" t="n"/>
       <c r="E11" s="7" t="n">
         <v>149.99</v>
       </c>
@@ -2409,7 +2397,7 @@
         </is>
       </c>
       <c r="K11" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L11" s="16">
         <f>IF(OR($K11="",D11=""),"",IF(COUNTIFS($B:$B,$B11,$A:$A,$K11,D:D,"&gt;=0")=0,"",D11-SUMIFS(D:D,$B:$B,$B11,$A:$A,$K11)))</f>
@@ -2430,7 +2418,7 @@
     </row>
     <row r="12">
       <c r="A12" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -2446,12 +2434,10 @@
         <v>150</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>119.95</v>
+        <v>99</v>
       </c>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="8" t="n">
-        <v>2460</v>
-      </c>
+      <c r="G12" s="2" t="n"/>
       <c r="H12" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A12,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A12,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2465,7 +2451,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K12" s="5" t="n"/>
+      <c r="K12" s="15" t="n">
+        <v>46307</v>
+      </c>
       <c r="L12" s="16">
         <f>IF(OR($K12="",D12=""),"",IF(COUNTIFS($B:$B,$B12,$A:$A,$K12,D:D,"&gt;=0")=0,"",D12-SUMIFS(D:D,$B:$B,$B12,$A:$A,$K12)))</f>
         <v/>
@@ -2485,7 +2473,7 @@
     </row>
     <row r="13">
       <c r="A13" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -2498,15 +2486,13 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>244.87</v>
+        <v>234.99</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>209.99</v>
       </c>
       <c r="F13" s="2" t="n"/>
-      <c r="G13" s="8" t="n">
-        <v>4290</v>
-      </c>
+      <c r="G13" s="2" t="n"/>
       <c r="H13" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A13,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A13,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2521,7 +2507,7 @@
         </is>
       </c>
       <c r="K13" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L13" s="16">
         <f>IF(OR($K13="",D13=""),"",IF(COUNTIFS($B:$B,$B13,$A:$A,$K13,D:D,"&gt;=0")=0,"",D13-SUMIFS(D:D,$B:$B,$B13,$A:$A,$K13)))</f>
@@ -2542,7 +2528,7 @@
     </row>
     <row r="14">
       <c r="A14" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
@@ -2576,7 +2562,7 @@
         </is>
       </c>
       <c r="K14" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="L14" s="16">
         <f>IF(OR($K14="",D14=""),"",IF(COUNTIFS($B:$B,$B14,$A:$A,$K14,D:D,"&gt;=0")=0,"",D14-SUMIFS(D:D,$B:$B,$B14,$A:$A,$K14)))</f>
@@ -2597,7 +2583,7 @@
     </row>
     <row r="15">
       <c r="A15" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
@@ -2613,11 +2599,9 @@
         <v>493</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>399.99</v>
-      </c>
-      <c r="F15" s="8" t="n">
-        <v>4500</v>
-      </c>
+        <v>383.99</v>
+      </c>
+      <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A15,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A15,Dólar!$A:$A,0))),"")</f>
@@ -2632,7 +2616,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K15" s="5" t="n"/>
+      <c r="K15" s="15" t="n">
+        <v>46307</v>
+      </c>
       <c r="L15" s="16">
         <f>IF(OR($K15="",D15=""),"",IF(COUNTIFS($B:$B,$B15,$A:$A,$K15,D:D,"&gt;=0")=0,"",D15-SUMIFS(D:D,$B:$B,$B15,$A:$A,$K15)))</f>
         <v/>
@@ -2652,7 +2638,7 @@
     </row>
     <row r="16">
       <c r="A16" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
@@ -2664,10 +2650,16 @@
           <t>SSD</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
+      <c r="D16" s="7" t="n">
+        <v>209.99</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>179.99</v>
+      </c>
       <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
+      <c r="G16" s="8" t="n">
+        <v>4060</v>
+      </c>
       <c r="H16" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A16,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A16,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2676,8 +2668,14 @@
         <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A16,Dólar!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="5" t="n"/>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K16" s="15" t="n">
+        <v>46306</v>
+      </c>
       <c r="L16" s="16">
         <f>IF(OR($K16="",D16=""),"",IF(COUNTIFS($B:$B,$B16,$A:$A,$K16,D:D,"&gt;=0")=0,"",D16-SUMIFS(D:D,$B:$B,$B16,$A:$A,$K16)))</f>
         <v/>
@@ -2697,7 +2695,7 @@
     </row>
     <row r="17">
       <c r="A17" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
@@ -2709,12 +2707,16 @@
           <t>SSD</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G17" s="2" t="n"/>
+      <c r="D17" s="7" t="n">
+        <v>114.99</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="8" t="n">
+        <v>1860</v>
+      </c>
       <c r="H17" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A17,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A17,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2728,7 +2730,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K17" s="5" t="n"/>
+      <c r="K17" s="15" t="n">
+        <v>46306</v>
+      </c>
       <c r="L17" s="16">
         <f>IF(OR($K17="",D17=""),"",IF(COUNTIFS($B:$B,$B17,$A:$A,$K17,D:D,"&gt;=0")=0,"",D17-SUMIFS(D:D,$B:$B,$B17,$A:$A,$K17)))</f>
         <v/>
@@ -2748,7 +2752,7 @@
     </row>
     <row r="18">
       <c r="A18" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
@@ -2760,11 +2764,15 @@
           <t>CPU</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
+      <c r="D18" s="7" t="n">
+        <v>499.99</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>454.99</v>
+      </c>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="8" t="n">
-        <v>5580</v>
+        <v>6140</v>
       </c>
       <c r="H18" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A18,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A18,Dólar!$A:$A,0))),"")</f>
@@ -2779,7 +2787,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K18" s="5" t="n"/>
+      <c r="K18" s="15" t="n">
+        <v>46306</v>
+      </c>
       <c r="L18" s="16">
         <f>IF(OR($K18="",D18=""),"",IF(COUNTIFS($B:$B,$B18,$A:$A,$K18,D:D,"&gt;=0")=0,"",D18-SUMIFS(D:D,$B:$B,$B18,$A:$A,$K18)))</f>
         <v/>
@@ -2799,7 +2809,7 @@
     </row>
     <row r="19">
       <c r="A19" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -2811,12 +2821,16 @@
           <t>CPU</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="8" t="n">
-        <v>4800</v>
-      </c>
-      <c r="G19" s="2" t="n"/>
+      <c r="D19" s="7" t="n">
+        <v>329</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>283.99</v>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="8" t="n">
+        <v>4760</v>
+      </c>
       <c r="H19" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A19,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A19,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2830,7 +2844,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K19" s="5" t="n"/>
+      <c r="K19" s="15" t="n">
+        <v>46306</v>
+      </c>
       <c r="L19" s="16">
         <f>IF(OR($K19="",D19=""),"",IF(COUNTIFS($B:$B,$B19,$A:$A,$K19,D:D,"&gt;=0")=0,"",D19-SUMIFS(D:D,$B:$B,$B19,$A:$A,$K19)))</f>
         <v/>
@@ -2850,11 +2866,11 @@
     </row>
     <row r="20">
       <c r="A20" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>Ryzen 7 5700X3D</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -2863,7 +2879,9 @@
         </is>
       </c>
       <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
+      <c r="E20" s="7" t="n">
+        <v>305</v>
+      </c>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="9">
@@ -2874,7 +2892,11 @@
         <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A20,Dólar!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="J20" s="2" t="n"/>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="16">
         <f>IF(OR($K20="",D20=""),"",IF(COUNTIFS($B:$B,$B20,$A:$A,$K20,D:D,"&gt;=0")=0,"",D20-SUMIFS(D:D,$B:$B,$B20,$A:$A,$K20)))</f>
@@ -2895,24 +2917,28 @@
     </row>
     <row r="21">
       <c r="A21" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR4 16GB (2x8) 3200</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>RAM</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="8" t="n">
-        <v>900</v>
-      </c>
-      <c r="G21" s="2" t="n"/>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>144.25</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>122.99</v>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="8" t="n">
+        <v>2860</v>
+      </c>
       <c r="H21" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A21,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A21,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2926,7 +2952,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K21" s="5" t="n"/>
+      <c r="K21" s="15" t="n">
+        <v>46306</v>
+      </c>
       <c r="L21" s="16">
         <f>IF(OR($K21="",D21=""),"",IF(COUNTIFS($B:$B,$B21,$A:$A,$K21,D:D,"&gt;=0")=0,"",D21-SUMIFS(D:D,$B:$B,$B21,$A:$A,$K21)))</f>
         <v/>
@@ -2946,11 +2974,11 @@
     </row>
     <row r="22">
       <c r="A22" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-14400F</t>
+          <t>Ryzen 5 5600</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2958,8 +2986,12 @@
           <t>CPU</t>
         </is>
       </c>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
+      <c r="D22" s="7" t="n">
+        <v>138.9</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>135</v>
+      </c>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="9">
@@ -2970,7 +3002,11 @@
         <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A22,Dólar!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="J22" s="2" t="n"/>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="16">
         <f>IF(OR($K22="",D22=""),"",IF(COUNTIFS($B:$B,$B22,$A:$A,$K22,D:D,"&gt;=0")=0,"",D22-SUMIFS(D:D,$B:$B,$B22,$A:$A,$K22)))</f>
@@ -2991,23 +3027,27 @@
     </row>
     <row r="23">
       <c r="A23" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-13400</t>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>59.99</v>
+      </c>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="8" t="n">
-        <v>2300</v>
+        <v>2150</v>
       </c>
       <c r="H23" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A23,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A23,Dólar!$A:$A,0))),"")</f>
@@ -3022,7 +3062,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K23" s="5" t="n"/>
+      <c r="K23" s="15" t="n">
+        <v>46306</v>
+      </c>
       <c r="L23" s="16">
         <f>IF(OR($K23="",D23=""),"",IF(COUNTIFS($B:$B,$B23,$A:$A,$K23,D:D,"&gt;=0")=0,"",D23-SUMIFS(D:D,$B:$B,$B23,$A:$A,$K23)))</f>
         <v/>
@@ -3042,11 +3084,11 @@
     </row>
     <row r="24">
       <c r="A24" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Intel Core Ultra 7 265K</t>
+          <t>Intel Core i5-14400F</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -3054,11 +3096,15 @@
           <t>CPU</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
+      <c r="D24" s="7" t="n">
+        <v>164.49</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>136.99</v>
+      </c>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="8" t="n">
-        <v>3950</v>
+        <v>2520</v>
       </c>
       <c r="H24" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A24,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A24,Dólar!$A:$A,0))),"")</f>
@@ -3073,7 +3119,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K24" s="5" t="n"/>
+      <c r="K24" s="15" t="n">
+        <v>46306</v>
+      </c>
       <c r="L24" s="16">
         <f>IF(OR($K24="",D24=""),"",IF(COUNTIFS($B:$B,$B24,$A:$A,$K24,D:D,"&gt;=0")=0,"",D24-SUMIFS(D:D,$B:$B,$B24,$A:$A,$K24)))</f>
         <v/>
@@ -3093,23 +3141,25 @@
     </row>
     <row r="25">
       <c r="A25" s="15" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+          <t>Intel Core i5-13400</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>RAM</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="8" t="n">
-        <v>6200</v>
-      </c>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>259.78</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A25,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A25,Dólar!$A:$A,0))),"")</f>
@@ -3124,7 +3174,9 @@
           <t>ver anuncio</t>
         </is>
       </c>
-      <c r="K25" s="5" t="n"/>
+      <c r="K25" s="15" t="n">
+        <v>46306</v>
+      </c>
       <c r="L25" s="16">
         <f>IF(OR($K25="",D25=""),"",IF(COUNTIFS($B:$B,$B25,$A:$A,$K25,D:D,"&gt;=0")=0,"",D25-SUMIFS(D:D,$B:$B,$B25,$A:$A,$K25)))</f>
         <v/>
@@ -3142,8 +3194,722 @@
         <v/>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-12400F</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>119.95</v>
+      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="8" t="n">
+        <v>2460</v>
+      </c>
+      <c r="H26" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A26,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A26,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A26,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="n"/>
+      <c r="L26" s="16">
+        <f>IF(OR($K26="",D26=""),"",IF(COUNTIFS($B:$B,$B26,$A:$A,$K26,D:D,"&gt;=0")=0,"",D26-SUMIFS(D:D,$B:$B,$B26,$A:$A,$K26)))</f>
+        <v/>
+      </c>
+      <c r="M26" s="16">
+        <f>IF(OR($K26="",E26=""),"",IF(COUNTIFS($B:$B,$B26,$A:$A,$K26,E:E,"&gt;=0")=0,"",E26-SUMIFS(E:E,$B:$B,$B26,$A:$A,$K26)))</f>
+        <v/>
+      </c>
+      <c r="N26" s="16">
+        <f>IF(OR($K26="",F26=""),"",IF(COUNTIFS($B:$B,$B26,$A:$A,$K26,F:F,"&gt;=0")=0,"",F26-SUMIFS(F:F,$B:$B,$B26,$A:$A,$K26)))</f>
+        <v/>
+      </c>
+      <c r="O26" s="16">
+        <f>IF(OR($K26="",G26=""),"",IF(COUNTIFS($B:$B,$B26,$A:$A,$K26,G:G,"&gt;=0")=0,"",G26-SUMIFS(G:G,$B:$B,$B26,$A:$A,$K26)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>244.87</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>209.99</v>
+      </c>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="8" t="n">
+        <v>4290</v>
+      </c>
+      <c r="H27" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A27,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A27,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A27,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K27" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="L27" s="16">
+        <f>IF(OR($K27="",D27=""),"",IF(COUNTIFS($B:$B,$B27,$A:$A,$K27,D:D,"&gt;=0")=0,"",D27-SUMIFS(D:D,$B:$B,$B27,$A:$A,$K27)))</f>
+        <v/>
+      </c>
+      <c r="M27" s="16">
+        <f>IF(OR($K27="",E27=""),"",IF(COUNTIFS($B:$B,$B27,$A:$A,$K27,E:E,"&gt;=0")=0,"",E27-SUMIFS(E:E,$B:$B,$B27,$A:$A,$K27)))</f>
+        <v/>
+      </c>
+      <c r="N27" s="16">
+        <f>IF(OR($K27="",F27=""),"",IF(COUNTIFS($B:$B,$B27,$A:$A,$K27,F:F,"&gt;=0")=0,"",F27-SUMIFS(F:F,$B:$B,$B27,$A:$A,$K27)))</f>
+        <v/>
+      </c>
+      <c r="O27" s="16">
+        <f>IF(OR($K27="",G27=""),"",IF(COUNTIFS($B:$B,$B27,$A:$A,$K27,G:G,"&gt;=0")=0,"",G27-SUMIFS(G:G,$B:$B,$B27,$A:$A,$K27)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>435.99</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>399.9</v>
+      </c>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A28,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A28,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A28,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K28" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="L28" s="16">
+        <f>IF(OR($K28="",D28=""),"",IF(COUNTIFS($B:$B,$B28,$A:$A,$K28,D:D,"&gt;=0")=0,"",D28-SUMIFS(D:D,$B:$B,$B28,$A:$A,$K28)))</f>
+        <v/>
+      </c>
+      <c r="M28" s="16">
+        <f>IF(OR($K28="",E28=""),"",IF(COUNTIFS($B:$B,$B28,$A:$A,$K28,E:E,"&gt;=0")=0,"",E28-SUMIFS(E:E,$B:$B,$B28,$A:$A,$K28)))</f>
+        <v/>
+      </c>
+      <c r="N28" s="16">
+        <f>IF(OR($K28="",F28=""),"",IF(COUNTIFS($B:$B,$B28,$A:$A,$K28,F:F,"&gt;=0")=0,"",F28-SUMIFS(F:F,$B:$B,$B28,$A:$A,$K28)))</f>
+        <v/>
+      </c>
+      <c r="O28" s="16">
+        <f>IF(OR($K28="",G28=""),"",IF(COUNTIFS($B:$B,$B28,$A:$A,$K28,G:G,"&gt;=0")=0,"",G28-SUMIFS(G:G,$B:$B,$B28,$A:$A,$K28)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>493</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>399.99</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A29,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A29,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A29,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="n"/>
+      <c r="L29" s="16">
+        <f>IF(OR($K29="",D29=""),"",IF(COUNTIFS($B:$B,$B29,$A:$A,$K29,D:D,"&gt;=0")=0,"",D29-SUMIFS(D:D,$B:$B,$B29,$A:$A,$K29)))</f>
+        <v/>
+      </c>
+      <c r="M29" s="16">
+        <f>IF(OR($K29="",E29=""),"",IF(COUNTIFS($B:$B,$B29,$A:$A,$K29,E:E,"&gt;=0")=0,"",E29-SUMIFS(E:E,$B:$B,$B29,$A:$A,$K29)))</f>
+        <v/>
+      </c>
+      <c r="N29" s="16">
+        <f>IF(OR($K29="",F29=""),"",IF(COUNTIFS($B:$B,$B29,$A:$A,$K29,F:F,"&gt;=0")=0,"",F29-SUMIFS(F:F,$B:$B,$B29,$A:$A,$K29)))</f>
+        <v/>
+      </c>
+      <c r="O29" s="16">
+        <f>IF(OR($K29="",G29=""),"",IF(COUNTIFS($B:$B,$B29,$A:$A,$K29,G:G,"&gt;=0")=0,"",G29-SUMIFS(G:G,$B:$B,$B29,$A:$A,$K29)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 2TB</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A30,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A30,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I30" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A30,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="5" t="n"/>
+      <c r="L30" s="16">
+        <f>IF(OR($K30="",D30=""),"",IF(COUNTIFS($B:$B,$B30,$A:$A,$K30,D:D,"&gt;=0")=0,"",D30-SUMIFS(D:D,$B:$B,$B30,$A:$A,$K30)))</f>
+        <v/>
+      </c>
+      <c r="M30" s="16">
+        <f>IF(OR($K30="",E30=""),"",IF(COUNTIFS($B:$B,$B30,$A:$A,$K30,E:E,"&gt;=0")=0,"",E30-SUMIFS(E:E,$B:$B,$B30,$A:$A,$K30)))</f>
+        <v/>
+      </c>
+      <c r="N30" s="16">
+        <f>IF(OR($K30="",F30=""),"",IF(COUNTIFS($B:$B,$B30,$A:$A,$K30,F:F,"&gt;=0")=0,"",F30-SUMIFS(F:F,$B:$B,$B30,$A:$A,$K30)))</f>
+        <v/>
+      </c>
+      <c r="O30" s="16">
+        <f>IF(OR($K30="",G30=""),"",IF(COUNTIFS($B:$B,$B30,$A:$A,$K30,G:G,"&gt;=0")=0,"",G30-SUMIFS(G:G,$B:$B,$B30,$A:$A,$K30)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="8" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A31,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A31,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I31" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A31,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="n"/>
+      <c r="L31" s="16">
+        <f>IF(OR($K31="",D31=""),"",IF(COUNTIFS($B:$B,$B31,$A:$A,$K31,D:D,"&gt;=0")=0,"",D31-SUMIFS(D:D,$B:$B,$B31,$A:$A,$K31)))</f>
+        <v/>
+      </c>
+      <c r="M31" s="16">
+        <f>IF(OR($K31="",E31=""),"",IF(COUNTIFS($B:$B,$B31,$A:$A,$K31,E:E,"&gt;=0")=0,"",E31-SUMIFS(E:E,$B:$B,$B31,$A:$A,$K31)))</f>
+        <v/>
+      </c>
+      <c r="N31" s="16">
+        <f>IF(OR($K31="",F31=""),"",IF(COUNTIFS($B:$B,$B31,$A:$A,$K31,F:F,"&gt;=0")=0,"",F31-SUMIFS(F:F,$B:$B,$B31,$A:$A,$K31)))</f>
+        <v/>
+      </c>
+      <c r="O31" s="16">
+        <f>IF(OR($K31="",G31=""),"",IF(COUNTIFS($B:$B,$B31,$A:$A,$K31,G:G,"&gt;=0")=0,"",G31-SUMIFS(G:G,$B:$B,$B31,$A:$A,$K31)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 9 9950X</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="8" t="n">
+        <v>5580</v>
+      </c>
+      <c r="H32" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A32,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A32,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A32,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="n"/>
+      <c r="L32" s="16">
+        <f>IF(OR($K32="",D32=""),"",IF(COUNTIFS($B:$B,$B32,$A:$A,$K32,D:D,"&gt;=0")=0,"",D32-SUMIFS(D:D,$B:$B,$B32,$A:$A,$K32)))</f>
+        <v/>
+      </c>
+      <c r="M32" s="16">
+        <f>IF(OR($K32="",E32=""),"",IF(COUNTIFS($B:$B,$B32,$A:$A,$K32,E:E,"&gt;=0")=0,"",E32-SUMIFS(E:E,$B:$B,$B32,$A:$A,$K32)))</f>
+        <v/>
+      </c>
+      <c r="N32" s="16">
+        <f>IF(OR($K32="",F32=""),"",IF(COUNTIFS($B:$B,$B32,$A:$A,$K32,F:F,"&gt;=0")=0,"",F32-SUMIFS(F:F,$B:$B,$B32,$A:$A,$K32)))</f>
+        <v/>
+      </c>
+      <c r="O32" s="16">
+        <f>IF(OR($K32="",G32=""),"",IF(COUNTIFS($B:$B,$B32,$A:$A,$K32,G:G,"&gt;=0")=0,"",G32-SUMIFS(G:G,$B:$B,$B32,$A:$A,$K32)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="8" t="n">
+        <v>4800</v>
+      </c>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A33,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A33,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I33" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A33,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="n"/>
+      <c r="L33" s="16">
+        <f>IF(OR($K33="",D33=""),"",IF(COUNTIFS($B:$B,$B33,$A:$A,$K33,D:D,"&gt;=0")=0,"",D33-SUMIFS(D:D,$B:$B,$B33,$A:$A,$K33)))</f>
+        <v/>
+      </c>
+      <c r="M33" s="16">
+        <f>IF(OR($K33="",E33=""),"",IF(COUNTIFS($B:$B,$B33,$A:$A,$K33,E:E,"&gt;=0")=0,"",E33-SUMIFS(E:E,$B:$B,$B33,$A:$A,$K33)))</f>
+        <v/>
+      </c>
+      <c r="N33" s="16">
+        <f>IF(OR($K33="",F33=""),"",IF(COUNTIFS($B:$B,$B33,$A:$A,$K33,F:F,"&gt;=0")=0,"",F33-SUMIFS(F:F,$B:$B,$B33,$A:$A,$K33)))</f>
+        <v/>
+      </c>
+      <c r="O33" s="16">
+        <f>IF(OR($K33="",G33=""),"",IF(COUNTIFS($B:$B,$B33,$A:$A,$K33,G:G,"&gt;=0")=0,"",G33-SUMIFS(G:G,$B:$B,$B33,$A:$A,$K33)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A34,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A34,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I34" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A34,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="5" t="n"/>
+      <c r="L34" s="16">
+        <f>IF(OR($K34="",D34=""),"",IF(COUNTIFS($B:$B,$B34,$A:$A,$K34,D:D,"&gt;=0")=0,"",D34-SUMIFS(D:D,$B:$B,$B34,$A:$A,$K34)))</f>
+        <v/>
+      </c>
+      <c r="M34" s="16">
+        <f>IF(OR($K34="",E34=""),"",IF(COUNTIFS($B:$B,$B34,$A:$A,$K34,E:E,"&gt;=0")=0,"",E34-SUMIFS(E:E,$B:$B,$B34,$A:$A,$K34)))</f>
+        <v/>
+      </c>
+      <c r="N34" s="16">
+        <f>IF(OR($K34="",F34=""),"",IF(COUNTIFS($B:$B,$B34,$A:$A,$K34,F:F,"&gt;=0")=0,"",F34-SUMIFS(F:F,$B:$B,$B34,$A:$A,$K34)))</f>
+        <v/>
+      </c>
+      <c r="O34" s="16">
+        <f>IF(OR($K34="",G34=""),"",IF(COUNTIFS($B:$B,$B34,$A:$A,$K34,G:G,"&gt;=0")=0,"",G34-SUMIFS(G:G,$B:$B,$B34,$A:$A,$K34)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="8" t="n">
+        <v>900</v>
+      </c>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A35,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A35,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I35" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A35,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="n"/>
+      <c r="L35" s="16">
+        <f>IF(OR($K35="",D35=""),"",IF(COUNTIFS($B:$B,$B35,$A:$A,$K35,D:D,"&gt;=0")=0,"",D35-SUMIFS(D:D,$B:$B,$B35,$A:$A,$K35)))</f>
+        <v/>
+      </c>
+      <c r="M35" s="16">
+        <f>IF(OR($K35="",E35=""),"",IF(COUNTIFS($B:$B,$B35,$A:$A,$K35,E:E,"&gt;=0")=0,"",E35-SUMIFS(E:E,$B:$B,$B35,$A:$A,$K35)))</f>
+        <v/>
+      </c>
+      <c r="N35" s="16">
+        <f>IF(OR($K35="",F35=""),"",IF(COUNTIFS($B:$B,$B35,$A:$A,$K35,F:F,"&gt;=0")=0,"",F35-SUMIFS(F:F,$B:$B,$B35,$A:$A,$K35)))</f>
+        <v/>
+      </c>
+      <c r="O35" s="16">
+        <f>IF(OR($K35="",G35=""),"",IF(COUNTIFS($B:$B,$B35,$A:$A,$K35,G:G,"&gt;=0")=0,"",G35-SUMIFS(G:G,$B:$B,$B35,$A:$A,$K35)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A36,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A36,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A36,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="5" t="n"/>
+      <c r="L36" s="16">
+        <f>IF(OR($K36="",D36=""),"",IF(COUNTIFS($B:$B,$B36,$A:$A,$K36,D:D,"&gt;=0")=0,"",D36-SUMIFS(D:D,$B:$B,$B36,$A:$A,$K36)))</f>
+        <v/>
+      </c>
+      <c r="M36" s="16">
+        <f>IF(OR($K36="",E36=""),"",IF(COUNTIFS($B:$B,$B36,$A:$A,$K36,E:E,"&gt;=0")=0,"",E36-SUMIFS(E:E,$B:$B,$B36,$A:$A,$K36)))</f>
+        <v/>
+      </c>
+      <c r="N36" s="16">
+        <f>IF(OR($K36="",F36=""),"",IF(COUNTIFS($B:$B,$B36,$A:$A,$K36,F:F,"&gt;=0")=0,"",F36-SUMIFS(F:F,$B:$B,$B36,$A:$A,$K36)))</f>
+        <v/>
+      </c>
+      <c r="O36" s="16">
+        <f>IF(OR($K36="",G36=""),"",IF(COUNTIFS($B:$B,$B36,$A:$A,$K36,G:G,"&gt;=0")=0,"",G36-SUMIFS(G:G,$B:$B,$B36,$A:$A,$K36)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-13400</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="8" t="n">
+        <v>2300</v>
+      </c>
+      <c r="H37" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A37,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A37,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A37,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="n"/>
+      <c r="L37" s="16">
+        <f>IF(OR($K37="",D37=""),"",IF(COUNTIFS($B:$B,$B37,$A:$A,$K37,D:D,"&gt;=0")=0,"",D37-SUMIFS(D:D,$B:$B,$B37,$A:$A,$K37)))</f>
+        <v/>
+      </c>
+      <c r="M37" s="16">
+        <f>IF(OR($K37="",E37=""),"",IF(COUNTIFS($B:$B,$B37,$A:$A,$K37,E:E,"&gt;=0")=0,"",E37-SUMIFS(E:E,$B:$B,$B37,$A:$A,$K37)))</f>
+        <v/>
+      </c>
+      <c r="N37" s="16">
+        <f>IF(OR($K37="",F37=""),"",IF(COUNTIFS($B:$B,$B37,$A:$A,$K37,F:F,"&gt;=0")=0,"",F37-SUMIFS(F:F,$B:$B,$B37,$A:$A,$K37)))</f>
+        <v/>
+      </c>
+      <c r="O37" s="16">
+        <f>IF(OR($K37="",G37=""),"",IF(COUNTIFS($B:$B,$B37,$A:$A,$K37,G:G,"&gt;=0")=0,"",G37-SUMIFS(G:G,$B:$B,$B37,$A:$A,$K37)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="8" t="n">
+        <v>3950</v>
+      </c>
+      <c r="H38" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A38,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A38,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A38,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="n"/>
+      <c r="L38" s="16">
+        <f>IF(OR($K38="",D38=""),"",IF(COUNTIFS($B:$B,$B38,$A:$A,$K38,D:D,"&gt;=0")=0,"",D38-SUMIFS(D:D,$B:$B,$B38,$A:$A,$K38)))</f>
+        <v/>
+      </c>
+      <c r="M38" s="16">
+        <f>IF(OR($K38="",E38=""),"",IF(COUNTIFS($B:$B,$B38,$A:$A,$K38,E:E,"&gt;=0")=0,"",E38-SUMIFS(E:E,$B:$B,$B38,$A:$A,$K38)))</f>
+        <v/>
+      </c>
+      <c r="N38" s="16">
+        <f>IF(OR($K38="",F38=""),"",IF(COUNTIFS($B:$B,$B38,$A:$A,$K38,F:F,"&gt;=0")=0,"",F38-SUMIFS(F:F,$B:$B,$B38,$A:$A,$K38)))</f>
+        <v/>
+      </c>
+      <c r="O38" s="16">
+        <f>IF(OR($K38="",G38=""),"",IF(COUNTIFS($B:$B,$B38,$A:$A,$K38,G:G,"&gt;=0")=0,"",G38-SUMIFS(G:G,$B:$B,$B38,$A:$A,$K38)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="8" t="n">
+        <v>6200</v>
+      </c>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="9">
+        <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A39,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A39,Dólar!$A:$A,0))),"")</f>
+        <v/>
+      </c>
+      <c r="I39" s="10">
+        <f>IFERROR(INDEX(Dólar!$E:$E,MATCH(A39,Dólar!$A:$A,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>ver anuncio</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="n"/>
+      <c r="L39" s="16">
+        <f>IF(OR($K39="",D39=""),"",IF(COUNTIFS($B:$B,$B39,$A:$A,$K39,D:D,"&gt;=0")=0,"",D39-SUMIFS(D:D,$B:$B,$B39,$A:$A,$K39)))</f>
+        <v/>
+      </c>
+      <c r="M39" s="16">
+        <f>IF(OR($K39="",E39=""),"",IF(COUNTIFS($B:$B,$B39,$A:$A,$K39,E:E,"&gt;=0")=0,"",E39-SUMIFS(E:E,$B:$B,$B39,$A:$A,$K39)))</f>
+        <v/>
+      </c>
+      <c r="N39" s="16">
+        <f>IF(OR($K39="",F39=""),"",IF(COUNTIFS($B:$B,$B39,$A:$A,$K39,F:F,"&gt;=0")=0,"",F39-SUMIFS(F:F,$B:$B,$B39,$A:$A,$K39)))</f>
+        <v/>
+      </c>
+      <c r="O39" s="16">
+        <f>IF(OR($K39="",G39=""),"",IF(COUNTIFS($B:$B,$B39,$A:$A,$K39,G:G,"&gt;=0")=0,"",G39-SUMIFS(G:G,$B:$B,$B39,$A:$A,$K39)))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="L2:M25">
+  <conditionalFormatting sqref="L2:M39">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -3151,7 +3917,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:O25">
+  <conditionalFormatting sqref="N2:O39">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3174,17 +3940,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId36"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3349,7 +4129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3470,6 +4250,32 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="E5" s="10">
+        <f>IF(COUNT(C5:D5)=2,AVERAGE(C5:D5),"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>BCB oficial 11.73; paralelo dolarbolivia.net 13/10 (compra 11.85 / venta 11.88); usado = promedio del paralelo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3481,7 +4287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H102"/>
+  <dimension ref="A1:H128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5552,34 +6358,34 @@
     </row>
     <row r="55">
       <c r="A55" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 9 9950X</t>
+          <t>Ryzen 5 5600</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>MSR Computers (web; fecha de actualización desconocida)</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E55" s="11" t="n">
-        <v>5580</v>
+        <v>138.9</v>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>eBay API; vendedor 3c_wholesaler 99.1%; (New) AMD Ryzen 5 5600 Vermeer Zen3 6-Core 12-Thread AM4 CPU</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
@@ -5590,34 +6396,34 @@
     </row>
     <row r="56">
       <c r="A56" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-13400</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>MSR Computers (web; fecha de actualización desconocida)</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E56" s="11" t="n">
-        <v>2300</v>
+        <v>143.24</v>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>eBay API; vendedor silaxon 99.6%; AMD Ryzen 5 7600 3.80GHz 6 Core 12 Thread AM5 100-000001015</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr">
@@ -5628,34 +6434,34 @@
     </row>
     <row r="57">
       <c r="A57" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Intel Core Ultra 7 265K</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>MSR Computers (web; fecha de actualización desconocida)</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E57" s="11" t="n">
-        <v>3950</v>
+        <v>329</v>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>nuevo</t>
+          <t>eBay API; vendedor aaawavecom 99.8%; AMD Ryzen 7 7800X3D Processor Zen 4 8-Core 4.2GHz AM5 CPU (N</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
@@ -5666,34 +6472,34 @@
     </row>
     <row r="58">
       <c r="A58" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Ryzen 9 9950X</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba (particular/vendedor)</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E58" s="11" t="n">
-        <v>4800</v>
+        <v>499.99</v>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>nuevo sellado (según anuncio)</t>
+          <t>eBay API; vendedor saguarowholesalesupply 100.0%; AMD Ryzen 9 9950X Desktop Processor AM5 New Sealed; envío no indicado</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
@@ -5704,34 +6510,34 @@
     </row>
     <row r="59">
       <c r="A59" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core i5-12400F</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E59" s="11" t="n">
-        <v>5190</v>
+        <v>150</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>no indicado</t>
+          <t>eBay API; vendedor algonz1137 100.0%; INTEL CPU Core i5-12400F / 6/12 / 2.5GHz / 6xxChipset / BX80; envío no indicado</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr">
@@ -5742,34 +6548,34 @@
     </row>
     <row r="60">
       <c r="A60" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core i5-14400F</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E60" s="11" t="n">
-        <v>5390</v>
+        <v>164.49</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>no indicado</t>
+          <t xml:space="preserve">eBay API; vendedor newegg 99.6%; Intel Core i5-14400F - Core i5 14th Gen Raptor Lake 10-Core </t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr">
@@ -5780,34 +6586,34 @@
     </row>
     <row r="61">
       <c r="A61" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>Intel Core Ultra 7 265K</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Marketplace La Paz</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E61" s="11" t="n">
-        <v>2000</v>
+        <v>234.99</v>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>no indicado (es 7600X; está en La Paz: solo referencia)</t>
+          <t>eBay API; vendedor good_neighbor_mercantile 99.4%; Intel Core Ultra 7 265K CPU Desktop Processor LGA 1851 20-Co</t>
         </is>
       </c>
       <c r="H61" s="6" t="inlineStr">
@@ -5818,34 +6624,34 @@
     </row>
     <row r="62">
       <c r="A62" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Marketplace La Paz</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E62" s="11" t="n">
-        <v>2650</v>
+        <v>493</v>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>no indicado (es 7600X; está en La Paz: solo referencia)</t>
+          <t xml:space="preserve">eBay API; vendedor blessshoppingshangrila 100.0%; New Corsair VENGEANCE 32GB (2x16GB) Memory DDR5-5600MHz RAM </t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr">
@@ -5856,34 +6662,34 @@
     </row>
     <row r="63">
       <c r="A63" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-14400F</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E63" s="11" t="n">
-        <v>2700</v>
+        <v>435.99</v>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>confirmado por Messenger el 12/10: es el i5-14400 con gráficos (no el F), nuevo en blíster, precio final Bs 2.700; no cuenta</t>
+          <t>eBay API; vendedor wojiapanpan_4 100.0%; Corsair Vengeance RGB RS 32GB 2x16GB DDR5 6000 CL38 AMD EXPO</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr">
@@ -5894,34 +6700,34 @@
     </row>
     <row r="64">
       <c r="A64" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E64" s="11" t="n">
-        <v>6200</v>
+        <v>92.98999999999999</v>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>no indicado (modelo RS)</t>
+          <t>eBay API; vendedor klolot3 100.0%; TeamGroup Vulcan Z 16GB (2x8GB) DDR4 3200 Desktop Gaming RAM; envío no indicado</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr">
@@ -5932,34 +6738,34 @@
     </row>
     <row r="65">
       <c r="A65" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR4 16GB (2x8) 3200</t>
+          <t>SSD NVMe 1TB</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E65" s="11" t="n">
-        <v>540</v>
+        <v>114.99</v>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>no indicado (Kingston Fury Beast RGB 16GB 3200; probablemente 1x16; no cuenta)</t>
+          <t>eBay API; vendedor gadgetworld03 99.0%; Derlar DN-850Q 1TB M.2 NVME PCIe 4.0 SSD - New</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr">
@@ -5970,34 +6776,34 @@
     </row>
     <row r="66">
       <c r="A66" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR4 16GB (2x8) 3200</t>
+          <t>SSD NVMe 2TB</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="E66" s="11" t="n">
-        <v>900</v>
+        <v>209.99</v>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>no indicado (16GB 3200; configuración no indicada)</t>
+          <t>eBay API; vendedor ram_technologies 100.0%; RAM Tech 2TB NVMe SSD Gen4 M.2 2280 | 5000MB/s Read 4500MB/s</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr">
@@ -6008,34 +6814,34 @@
     </row>
     <row r="67">
       <c r="A67" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR4 16GB (2x8) 3200</t>
+          <t>Ryzen 5 5600</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E67" s="11" t="n">
-        <v>1500</v>
+        <v>135</v>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>no indicado (2x8 3200; Sacaba)</t>
+          <t>eBay API; vendedor btlsln 100.0%; AMD Ryzen 5 5600 Desktop Processor (6 Cores, Socket AM4); envío no indicado</t>
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr">
@@ -6046,34 +6852,34 @@
     </row>
     <row r="68">
       <c r="A68" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR4 16GB (2x8) 3200</t>
+          <t>Ryzen 7 5700X3D</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E68" s="11" t="n">
-        <v>1500</v>
+        <v>299.99</v>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>no indicado (Corsair Vengeance 2x8; Sacaba; rebajado de 1600)</t>
+          <t>eBay API; vendedor paymore_fontana 99.3%; AMD Ryzen 7 5700X3D 3.00GHz 8 Core 100-000001503 16 Thread A</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
@@ -6084,34 +6890,34 @@
     </row>
     <row r="69">
       <c r="A69" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E69" s="11" t="n">
-        <v>1850</v>
+        <v>122.99</v>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>no indicado (Kingston NV3 1TB)</t>
+          <t>eBay API; vendedor paymore_cumberland 98.6%; AMD Ryzen 5 7600 3.80GHz 6 Core 100-000001015 12 Thread AM5</t>
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr">
@@ -6122,34 +6928,34 @@
     </row>
     <row r="70">
       <c r="A70" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E70" s="11" t="n">
-        <v>2000</v>
+        <v>283.99</v>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>no indicado (Crucial P310 1TB)</t>
+          <t>eBay API; vendedor paymore_pooler 99.7%; AMD Ryzen 7 7800X3D 4.20GHz 8 Core 100-000000910 16 Thread A</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
@@ -6160,34 +6966,34 @@
     </row>
     <row r="71">
       <c r="A71" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Ryzen 9 9950X</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E71" s="11" t="n">
-        <v>1800</v>
+        <v>454.99</v>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>no indicado (M.2 1TB; marca no indicada)</t>
+          <t>eBay API; vendedor goodios_direct 99.6%; **  AMD Ryzen 9 9950X Processor - USED  **</t>
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr">
@@ -6198,34 +7004,34 @@
     </row>
     <row r="72">
       <c r="A72" s="15" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 2TB</t>
+          <t>Intel Core i5-12400F</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E72" s="11" t="n">
-        <v>3550</v>
+        <v>99</v>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>revisado el 12/10: es un SSD externo portátil SanDisk 2TB (1050 MB/s, USB con cable, IP65), no un NVMe interno; no cuenta</t>
+          <t>eBay API; vendedor sale_of_the_day 100.0%; Intel Core i5-12400F; envío no indicado</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
@@ -6236,34 +7042,34 @@
     </row>
     <row r="73">
       <c r="A73" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core i5-13400</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>Cyrex Store (WhatsApp)</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E73" s="11" t="n">
-        <v>5664</v>
+        <v>149.99</v>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>BOX (según foto de su web; USD 480)</t>
+          <t>eBay API; vendedor techrec-recycling 99.6%; Intel Core i5-13400 2.50GHz 10-Core LGA1700 20MB Desktop Pro</t>
         </is>
       </c>
       <c r="H73" s="6" t="inlineStr">
@@ -6274,11 +7080,11 @@
     </row>
     <row r="74">
       <c r="A74" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
@@ -6288,20 +7094,20 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Cyrex Store (WhatsApp)</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E74" s="11" t="n">
-        <v>2537</v>
+        <v>134</v>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>OEM (sin caja; según foto de su web; USD 215)</t>
+          <t>eBay API; vendedor htam86 99.7%; Intel Core i5-14400F 10-Core 16-Thread 4.7GHz LGA 1700 CPU S</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr">
@@ -6312,34 +7118,34 @@
     </row>
     <row r="75">
       <c r="A75" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR5 16GB (1x16) 6000</t>
+          <t>Intel Core Ultra 7 265K</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Cyrex Store (WhatsApp)</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E75" s="11" t="n">
-        <v>3127</v>
+        <v>209.99</v>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>no indicado (Patriot Viper Venom RGB 1x16 CL30; USD 265; no es el kit Corsair 2x16: solo referencia)</t>
+          <t xml:space="preserve">eBay API; vendedor paymore_bustleton 99.4%; Intel Core Ultra 7 265K 3.90GHz 20 Core SRQCW 20 Thread LGA </t>
         </is>
       </c>
       <c r="H75" s="6" t="inlineStr">
@@ -6350,34 +7156,34 @@
     </row>
     <row r="76">
       <c r="A76" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>RAM DDR4 16GB (2x8) 3200</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Compucenter (WhatsApp)</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E76" s="11" t="n">
-        <v>2150</v>
+        <v>383.99</v>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>nuevo (Corsair Vengeance RGB DDR4 16GB 3600; no dice si es 2x8; Bs 2.560 con factura)</t>
+          <t>eBay API; vendedor sly-systems 99.7%; Corsair Vengeance RGB Pro 32GB (2x16GB) RAM DDR5 5600MHz</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr">
@@ -6388,34 +7194,34 @@
     </row>
     <row r="77">
       <c r="A77" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 9 9950X</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Tienda Supermall (WhatsApp)</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E77" s="11" t="n">
-        <v>6140</v>
+        <v>399.9</v>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>nuevo OEM (garantía 6 meses)</t>
+          <t>eBay API; vendedor thaigamer 100.0%; Corsair Vengeance RGB DDR5 32GB (2x16GB) 6000MHz DIMM RGB CM; envío no indicado</t>
         </is>
       </c>
       <c r="H77" s="6" t="inlineStr">
@@ -6426,34 +7232,34 @@
     </row>
     <row r="78">
       <c r="A78" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Tienda Supermall (WhatsApp)</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E78" s="11" t="n">
-        <v>4760</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>no indicado (la tienda lo ofrece como "7700x3d"; foto de caja 7800X3D; stock bajo; garantía 6 meses; confirmar modelo)</t>
+          <t>eBay API; vendedor corefoundry 100.0%; ADATA XPG Spectrix D41 16GB (2x8GB) DDR4 3200MHz CL16 Deskto; envío no indicado</t>
         </is>
       </c>
       <c r="H78" s="6" t="inlineStr">
@@ -6464,34 +7270,34 @@
     </row>
     <row r="79">
       <c r="A79" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+          <t>SSD NVMe 1TB</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E79" s="11" t="n">
-        <v>6800</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>no indicado</t>
+          <t>eBay API; vendedor anotherdudestreasures 98.9%; SK hynix PC611 1TB NVMe PCIe Gen3 x4 M.2 2280 Internal SSD H</t>
         </is>
       </c>
       <c r="H79" s="6" t="inlineStr">
@@ -6502,34 +7308,34 @@
     </row>
     <row r="80">
       <c r="A80" s="15" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>SSD NVMe 2TB</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+          <t>usado</t>
         </is>
       </c>
       <c r="E80" s="11" t="n">
-        <v>2100</v>
+        <v>170</v>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Bs</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>no indicado (Kingston NV3 PCIe 4.0; Santa Cruz: referencia)</t>
+          <t>eBay API; vendedor bunyip1992 100.0%; Inland 2TB Gen 3 NVME SSD Used Good</t>
         </is>
       </c>
       <c r="H80" s="6" t="inlineStr">
@@ -6540,7 +7346,7 @@
     </row>
     <row r="81">
       <c r="A81" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
@@ -6549,16 +7355,16 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Ryzen 9 9950X</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+          <t>MSR Computers (web; fecha de actualización desconocida)</t>
         </is>
       </c>
       <c r="E81" s="11" t="n">
-        <v>1800</v>
+        <v>5580</v>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
@@ -6567,7 +7373,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>no indicado (marca "ediloca" PCIe 4.0; Santa Cruz: referencia)</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="H81" s="6" t="inlineStr">
@@ -6578,25 +7384,25 @@
     </row>
     <row r="82">
       <c r="A82" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Tienda</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+          <t>Intel Core i5-13400</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Cochabamba (particular)</t>
+          <t>MSR Computers (web; fecha de actualización desconocida)</t>
         </is>
       </c>
       <c r="E82" s="11" t="n">
-        <v>4500</v>
+        <v>2300</v>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
@@ -6605,7 +7411,7 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>usado como nuevo (4 meses de uso; publicado hace 7 semanas)</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr">
@@ -6616,7 +7422,7 @@
     </row>
     <row r="83">
       <c r="A83" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
@@ -6625,16 +7431,16 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+          <t>Intel Core Ultra 7 265K</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+          <t>MSR Computers (web; fecha de actualización desconocida)</t>
         </is>
       </c>
       <c r="E83" s="11" t="n">
-        <v>6700</v>
+        <v>3950</v>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
@@ -6643,7 +7449,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>no indicado (precio c/u llevando 2; Santa Cruz: referencia)</t>
+          <t>nuevo</t>
         </is>
       </c>
       <c r="H83" s="6" t="inlineStr">
@@ -6654,25 +7460,25 @@
     </row>
     <row r="84">
       <c r="A84" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-14400F</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba (particular/vendedor)</t>
         </is>
       </c>
       <c r="E84" s="11" t="n">
-        <v>2520</v>
+        <v>4800</v>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
@@ -6681,7 +7487,7 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>disponible (web)</t>
+          <t>nuevo sellado (según anuncio)</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
@@ -6692,25 +7498,25 @@
     </row>
     <row r="85">
       <c r="A85" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Intel Core Ultra 7 265K</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E85" s="11" t="n">
-        <v>4290</v>
+        <v>5190</v>
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
@@ -6719,7 +7525,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>stock bajo (web; por WhatsApp dijeron que el 265K solo está en Santa Cruz)</t>
+          <t>no indicado</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr">
@@ -6730,25 +7536,25 @@
     </row>
     <row r="86">
       <c r="A86" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E86" s="11" t="n">
-        <v>2860</v>
+        <v>5390</v>
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
@@ -6757,7 +7563,7 @@
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>stock bajo (web)</t>
+          <t>no indicado</t>
         </is>
       </c>
       <c r="H86" s="6" t="inlineStr">
@@ -6768,25 +7574,25 @@
     </row>
     <row r="87">
       <c r="A87" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-12400F</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace La Paz</t>
         </is>
       </c>
       <c r="E87" s="11" t="n">
-        <v>2460</v>
+        <v>2000</v>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
@@ -6795,7 +7601,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>disponible (web)</t>
+          <t>no indicado (es 7600X; está en La Paz: solo referencia)</t>
         </is>
       </c>
       <c r="H87" s="6" t="inlineStr">
@@ -6806,25 +7612,25 @@
     </row>
     <row r="88">
       <c r="A88" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace La Paz</t>
         </is>
       </c>
       <c r="E88" s="11" t="n">
-        <v>5360</v>
+        <v>2650</v>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
@@ -6833,7 +7639,7 @@
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>agotado (web, "Ryzen 7 7800x3d Chip"; precio de referencia; no cuenta)</t>
+          <t>no indicado (es 7600X; está en La Paz: solo referencia)</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
@@ -6844,25 +7650,25 @@
     </row>
     <row r="89">
       <c r="A89" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 5600</t>
+          <t>Intel Core i5-14400F</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E89" s="11" t="n">
-        <v>1710</v>
+        <v>2700</v>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
@@ -6871,7 +7677,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>agotado (web; precio de referencia; no cuenta)</t>
+          <t>confirmado por Messenger el 12/10: es el i5-14400 con gráficos (no el F), nuevo en blíster, precio final Bs 2.700; no cuenta</t>
         </is>
       </c>
       <c r="H89" s="6" t="inlineStr">
@@ -6882,25 +7688,25 @@
     </row>
     <row r="90">
       <c r="A90" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-13400</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E90" s="11" t="n">
-        <v>2310</v>
+        <v>6200</v>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
@@ -6909,7 +7715,7 @@
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>agotado (web; precio de referencia; no cuenta)</t>
+          <t>no indicado (modelo RS)</t>
         </is>
       </c>
       <c r="H90" s="6" t="inlineStr">
@@ -6920,11 +7726,11 @@
     </row>
     <row r="91">
       <c r="A91" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
@@ -6934,11 +7740,11 @@
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E91" s="11" t="n">
-        <v>2160</v>
+        <v>540</v>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
@@ -6947,7 +7753,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>disponible (web; Corsair Vengeance RGB Pro TUF Gaming 2x8 3200)</t>
+          <t>no indicado (Kingston Fury Beast RGB 16GB 3200; probablemente 1x16; no cuenta)</t>
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr">
@@ -6958,25 +7764,25 @@
     </row>
     <row r="92">
       <c r="A92" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E92" s="11" t="n">
-        <v>5360</v>
+        <v>900</v>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
@@ -6985,7 +7791,7 @@
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>agotado (web; precio de referencia; no cuenta)</t>
+          <t>no indicado (16GB 3200; configuración no indicada)</t>
         </is>
       </c>
       <c r="H92" s="6" t="inlineStr">
@@ -6996,25 +7802,25 @@
     </row>
     <row r="93">
       <c r="A93" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E93" s="11" t="n">
-        <v>5660</v>
+        <v>1500</v>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
@@ -7023,7 +7829,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>disponible (web; Patriot Viper 32GB 6000 RGB: otra marca; no cuenta)</t>
+          <t>no indicado (2x8 3200; Sacaba)</t>
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr">
@@ -7034,25 +7840,25 @@
     </row>
     <row r="94">
       <c r="A94" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E94" s="11" t="n">
-        <v>5860</v>
+        <v>1500</v>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
@@ -7061,7 +7867,7 @@
       </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
-          <t>disponible (web; Kingston Fury 32GB 2x16 5200/5600: otra marca; no cuenta)</t>
+          <t>no indicado (Corsair Vengeance 2x8; Sacaba; rebajado de 1600)</t>
         </is>
       </c>
       <c r="H94" s="6" t="inlineStr">
@@ -7072,11 +7878,11 @@
     </row>
     <row r="95">
       <c r="A95" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
@@ -7086,11 +7892,11 @@
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E95" s="11" t="n">
-        <v>1860</v>
+        <v>1850</v>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
@@ -7099,7 +7905,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>stock bajo (web; Hiksemi Wave M.2 1TB)</t>
+          <t>no indicado (Kingston NV3 1TB)</t>
         </is>
       </c>
       <c r="H95" s="6" t="inlineStr">
@@ -7110,11 +7916,11 @@
     </row>
     <row r="96">
       <c r="A96" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
@@ -7124,11 +7930,11 @@
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E96" s="11" t="n">
-        <v>2060</v>
+        <v>2000</v>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
@@ -7137,7 +7943,7 @@
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>disponible (web; WD SN3000 M.2 1TB)</t>
+          <t>no indicado (Crucial P310 1TB)</t>
         </is>
       </c>
       <c r="H96" s="6" t="inlineStr">
@@ -7148,11 +7954,11 @@
     </row>
     <row r="97">
       <c r="A97" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
@@ -7162,11 +7968,11 @@
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E97" s="11" t="n">
-        <v>2152</v>
+        <v>1800</v>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
@@ -7175,7 +7981,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>disponible (web; Kingston NV3 M.2 1TB)</t>
+          <t>no indicado (M.2 1TB; marca no indicada)</t>
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr">
@@ -7186,11 +7992,11 @@
     </row>
     <row r="98">
       <c r="A98" s="15" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>Tienda</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
@@ -7200,11 +8006,11 @@
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Marketplace Cochabamba</t>
         </is>
       </c>
       <c r="E98" s="11" t="n">
-        <v>4060</v>
+        <v>3550</v>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
@@ -7213,7 +8019,7 @@
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>stock bajo (web; Apacer M.2 2TB 7400 MB/s)</t>
+          <t>revisado el 12/10: es un SSD externo portátil SanDisk 2TB (1050 MB/s, USB con cable, IP65), no un NVMe interno; no cuenta</t>
         </is>
       </c>
       <c r="H98" s="6" t="inlineStr">
@@ -7233,16 +8039,16 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 2TB</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>Punto Tecnológico · Supermall (web)</t>
+          <t>Cyrex Store (WhatsApp)</t>
         </is>
       </c>
       <c r="E99" s="11" t="n">
-        <v>4560</v>
+        <v>5664</v>
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
@@ -7251,7 +8057,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>disponible (web; Hiksemi Futurex M.2 2TB)</t>
+          <t>BOX (según foto de su web; USD 480)</t>
         </is>
       </c>
       <c r="H99" s="6" t="inlineStr">
@@ -7271,16 +8077,16 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core i5-14400F</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>Viadata Computadoras (WhatsApp)</t>
+          <t>Cyrex Store (WhatsApp)</t>
         </is>
       </c>
       <c r="E100" s="11" t="n">
-        <v>5500</v>
+        <v>2537</v>
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
@@ -7289,7 +8095,7 @@
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>nuevo OEM (solo el chip)</t>
+          <t>OEM (sin caja; según foto de su web; USD 215)</t>
         </is>
       </c>
       <c r="H100" s="6" t="inlineStr">
@@ -7309,16 +8115,16 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 5600</t>
+          <t>RAM DDR5 16GB (1x16) 6000</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Viadata Computadoras (WhatsApp)</t>
+          <t>Cyrex Store (WhatsApp)</t>
         </is>
       </c>
       <c r="E101" s="11" t="n">
-        <v>2500</v>
+        <v>3127</v>
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
@@ -7327,7 +8133,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>nuevo OEM (es el 5600X, no el 5600; solo referencia; no cuenta)</t>
+          <t>no indicado (Patriot Viper Venom RGB 1x16 CL30; USD 265; no es el kit Corsair 2x16: solo referencia)</t>
         </is>
       </c>
       <c r="H101" s="6" t="inlineStr">
@@ -7347,28 +8153,1016 @@
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Compucenter (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E102" s="11" t="n">
+        <v>2150</v>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (Corsair Vengeance RGB DDR4 16GB 3600; no dice si es 2x8; Bs 2.560 con factura)</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 9 9950X</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>Tienda Supermall (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E103" s="11" t="n">
+        <v>6140</v>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (garantía 6 meses)</t>
+        </is>
+      </c>
+      <c r="H103" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D104" s="5" t="inlineStr">
+        <is>
+          <t>Tienda Supermall (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E104" s="11" t="n">
+        <v>4760</v>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (la tienda lo ofrece como "7700x3d"; foto de caja 7800X3D; stock bajo; garantía 6 meses; confirmar modelo)</t>
+        </is>
+      </c>
+      <c r="H104" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="E105" s="11" t="n">
+        <v>6800</v>
+      </c>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>no indicado</t>
+        </is>
+      </c>
+      <c r="H105" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="inlineStr">
+        <is>
+          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="E106" s="11" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (Kingston NV3 PCIe 4.0; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="E107" s="11" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (marca "ediloca" PCIe 4.0; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E108" s="11" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>usado como nuevo (4 meses de uso; publicado hace 7 semanas)</t>
+        </is>
+      </c>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>PC Components Bolivia (WhatsApp; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="E109" s="11" t="n">
+        <v>6700</v>
+      </c>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (precio c/u llevando 2; Santa Cruz: referencia)</t>
+        </is>
+      </c>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D110" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E110" s="11" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web)</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
           <t>Intel Core Ultra 7 265K</t>
         </is>
       </c>
-      <c r="D102" s="5" t="inlineStr">
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E111" s="11" t="n">
+        <v>4290</v>
+      </c>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>stock bajo (web; por WhatsApp dijeron que el 265K solo está en Santa Cruz)</t>
+        </is>
+      </c>
+      <c r="H111" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E112" s="11" t="n">
+        <v>2860</v>
+      </c>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>stock bajo (web)</t>
+        </is>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-12400F</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E113" s="11" t="n">
+        <v>2460</v>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web)</t>
+        </is>
+      </c>
+      <c r="H113" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E114" s="11" t="n">
+        <v>5360</v>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>agotado (web, "Ryzen 7 7800x3d Chip"; precio de referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 5600</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E115" s="11" t="n">
+        <v>1710</v>
+      </c>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>agotado (web; precio de referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H115" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-13400</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E116" s="11" t="n">
+        <v>2310</v>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>agotado (web; precio de referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E117" s="11" t="n">
+        <v>2160</v>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Corsair Vengeance RGB Pro TUF Gaming 2x8 3200)</t>
+        </is>
+      </c>
+      <c r="H117" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E118" s="11" t="n">
+        <v>5360</v>
+      </c>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
+          <t>agotado (web; precio de referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H118" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E119" s="11" t="n">
+        <v>5660</v>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Patriot Viper 32GB 6000 RGB: otra marca; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H119" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E120" s="11" t="n">
+        <v>5860</v>
+      </c>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G120" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Kingston Fury 32GB 2x16 5200/5600: otra marca; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H120" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E121" s="11" t="n">
+        <v>1860</v>
+      </c>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>stock bajo (web; Hiksemi Wave M.2 1TB)</t>
+        </is>
+      </c>
+      <c r="H121" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D122" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E122" s="11" t="n">
+        <v>2060</v>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; WD SN3000 M.2 1TB)</t>
+        </is>
+      </c>
+      <c r="H122" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E123" s="11" t="n">
+        <v>2152</v>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Kingston NV3 M.2 1TB)</t>
+        </is>
+      </c>
+      <c r="H123" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 2TB</t>
+        </is>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E124" s="11" t="n">
+        <v>4060</v>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
+          <t>stock bajo (web; Apacer M.2 2TB 7400 MB/s)</t>
+        </is>
+      </c>
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 2TB</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web)</t>
+        </is>
+      </c>
+      <c r="E125" s="11" t="n">
+        <v>4560</v>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; Hiksemi Futurex M.2 2TB)</t>
+        </is>
+      </c>
+      <c r="H125" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
         <is>
           <t>Viadata Computadoras (WhatsApp)</t>
         </is>
       </c>
-      <c r="E102" s="11" t="n">
+      <c r="E126" s="11" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (solo el chip)</t>
+        </is>
+      </c>
+      <c r="H126" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 5600</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>Viadata Computadoras (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E127" s="11" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (es el 5600X, no el 5600; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H127" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="15" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="D128" s="5" t="inlineStr">
+        <is>
+          <t>Viadata Computadoras (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E128" s="11" t="n">
         <v>5200</v>
       </c>
-      <c r="F102" s="5" t="inlineStr">
+      <c r="F128" s="5" t="inlineStr">
         <is>
           <t>Bs</t>
         </is>
       </c>
-      <c r="G102" s="5" t="inlineStr">
+      <c r="G128" s="5" t="inlineStr">
         <is>
           <t>nuevo en caja (es el 265KF, sin gráficos integrados; solo referencia; no cuenta)</t>
         </is>
       </c>
-      <c r="H102" s="6" t="inlineStr">
+      <c r="H128" s="6" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -7477,10 +9271,36 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId127"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId102"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId128"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
PC ronda de la tarde 13/10: precios de OverCity y Soft Computers, Messenger 7800X3D, rastreo de 3 pedidos de prueba (GOFO entregado en Miami), mapa con Carteret, Doral y Miami
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H128" headerRowCount="1">
-  <autoFilter ref="A1:H128"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H131" headerRowCount="1">
+  <autoFilter ref="A1:H131"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -1045,12 +1045,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-14400F</t>
+          <t>SSD NVMe 1TB</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1059,17 +1059,19 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>164.49</v>
+        <v>114.99</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>134</v>
-      </c>
-      <c r="G9" s="2" t="n"/>
+        <v>99.98999999999999</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>1800</v>
+      </c>
       <c r="H9" s="8" t="n">
-        <v>2520</v>
+        <v>1860</v>
       </c>
       <c r="I9" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1080,7 +1082,7 @@
         <v/>
       </c>
       <c r="K9" s="8" t="n">
-        <v>250</v>
+        <v>80</v>
       </c>
       <c r="L9" s="11">
         <f>IF(D9="","",MIN(MAX(Supuestos!$B$5,CEILING((K9*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D9*Supuestos!$B$9))</f>
@@ -1110,12 +1112,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1124,19 +1126,19 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>114.99</v>
+        <v>329</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>99.98999999999999</v>
+        <v>283.99</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>1800</v>
+        <v>4800</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>1860</v>
+        <v>4760</v>
       </c>
       <c r="I10" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1147,7 +1149,7 @@
         <v/>
       </c>
       <c r="K10" s="8" t="n">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="L10" s="11">
         <f>IF(D10="","",MIN(MAX(Supuestos!$B$5,CEILING((K10*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D10*Supuestos!$B$9))</f>
@@ -1177,7 +1179,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core i5-14400F</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1191,19 +1193,17 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>329</v>
+        <v>164.49</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>283.99</v>
-      </c>
-      <c r="G11" s="8" t="n">
-        <v>4800</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="G11" s="2" t="n"/>
       <c r="H11" s="8" t="n">
-        <v>4760</v>
+        <v>2460</v>
       </c>
       <c r="I11" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K11" s="8" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="L11" s="11">
         <f>IF(D11="","",MIN(MAX(Supuestos!$B$5,CEILING((K11*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D11*Supuestos!$B$9))</f>
@@ -2056,7 +2056,9 @@
         <v>283.99</v>
       </c>
       <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="8" t="n">
+        <v>5500</v>
+      </c>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2329,7 +2331,9 @@
         <v>134</v>
       </c>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
+      <c r="G10" s="8" t="n">
+        <v>2460</v>
+      </c>
       <c r="H10" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -4287,7 +4291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H128"/>
+  <dimension ref="A1:H131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9167,6 +9171,108 @@
           <t>ver</t>
         </is>
       </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="15" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>OverCity (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E129" s="11" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G129" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (solo el chip)</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="15" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>OverCity (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E130" s="11" t="n">
+        <v>2460</v>
+      </c>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G130" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="15" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>Soft Computers (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E131" s="11" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G131" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Aduana incluida en los dos couriers (confirmado por Santi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017XwuV2NE7bTCMuMMt3PVuA
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Historial" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -240,7 +240,7 @@
   <commentList>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>Aduana sin confirmar con los couriers: probar aquí, por ejemplo 0,1 = 10 %.</t>
+        <t>Los dos couriers ya incluyen la aduana (Santi, 13/10): queda en 0. Probar aquí solo si algún envío la cobra aparte, por ejemplo 0,1 = 10 %.</t>
       </text>
     </comment>
     <comment ref="B11" authorId="0" shapeId="0">
@@ -4071,7 +4071,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Aduana boliviana (sin confirmar)</t>
+          <t>Aduana boliviana extra (incluida en los couriers)</t>
         </is>
       </c>
       <c r="B10" s="22" t="n">

</xml_diff>

<commit_message>
Ronda Mac 13/10 tarde: actividad, métricas, comparación, Excel, captura de Marketplace y oficina publicada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Historial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H131" headerRowCount="1">
-  <autoFilter ref="A1:H131"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H133" headerRowCount="1">
+  <autoFilter ref="A1:H133"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2055,7 +2055,9 @@
       <c r="E5" s="7" t="n">
         <v>283.99</v>
       </c>
-      <c r="F5" s="2" t="n"/>
+      <c r="F5" s="8" t="n">
+        <v>4800</v>
+      </c>
       <c r="G5" s="8" t="n">
         <v>5500</v>
       </c>
@@ -4291,7 +4293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H131"/>
+  <dimension ref="A1:H133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9273,6 +9275,78 @@
         </is>
       </c>
       <c r="H131" s="2" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="15" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D132" s="5" t="inlineStr">
+        <is>
+          <t>OverCity (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E132" s="11" t="n">
+        <v>6840</v>
+      </c>
+      <c r="F132" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G132" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (XPG Lancer RGB 32GB 2x16 6000 CL30: otra marca; no cuenta; Corsair agotada; garantía 3 meses)</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="15" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular/vendedor; Messenger)</t>
+        </is>
+      </c>
+      <c r="E133" s="11" t="n">
+        <v>4800</v>
+      </c>
+      <c r="F133" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>nuevo sellado de fábrica, confirmado por el vendedor (último en stock; precio ya rebajado)</t>
+        </is>
+      </c>
+      <c r="H133" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -9403,10 +9477,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId128"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId128"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId129"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Posibles clientes a futuro (clientes-potenciales.csv); OverCity 7800X3D sellado Bs 5.350; eBay sin compras
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H133" headerRowCount="1">
-  <autoFilter ref="A1:H133"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H134" headerRowCount="1">
+  <autoFilter ref="A1:H134"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2059,7 +2059,7 @@
         <v>4800</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>5500</v>
+        <v>5350</v>
       </c>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
@@ -4293,7 +4293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H133"/>
+  <dimension ref="A1:H134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9347,6 +9347,40 @@
           <t>ver</t>
         </is>
       </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="15" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>OverCity (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E134" s="11" t="n">
+        <v>5350</v>
+      </c>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G134" s="5" t="inlineStr">
+        <is>
+          <t>nuevo en caja sellada (box; el OEM está a Bs 5.500; el i5-14400F Bs 2.460 es su precio mínimo)</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ronda Mac 14/10 mañana: 5 seguimientos, PC Factor y Crazy Store, TecnoGamer a grupo D, Marketplace y web de Geek Store, pedidos sin cambios, oficina publicada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historial" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Historial" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dólar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Movimientos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H160" headerRowCount="1">
-  <autoFilter ref="A1:H160"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H163" headerRowCount="1">
+  <autoFilter ref="A1:H163"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -5099,7 +5099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11175,6 +11175,116 @@
         </is>
       </c>
       <c r="H160" s="2" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="15" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba</t>
+        </is>
+      </c>
+      <c r="E161" s="11" t="n">
+        <v>7400</v>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="inlineStr">
+        <is>
+          <t>no indicado (Kingston Fury Beast DDR5 32GB 5600: otra marca; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H161" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="15" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>Geek Store Bolivia (web)</t>
+        </is>
+      </c>
+      <c r="E162" s="11" t="n">
+        <v>2953</v>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G162" s="5" t="inlineStr">
+        <is>
+          <t>disponible (web; es el i5-14400 con gráficos, no el F; precio USD 249 en la web, a Bs 11,86; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H162" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="15" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i9-14900K</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>Crazy Store (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E163" s="11" t="n">
+        <v>6013</v>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G163" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (no está en vigilar.csv; USD 499 o Bs 6.013, rebaja ofrecida hasta Bs 5.700; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11332,10 +11442,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H153" r:id="rId152"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H154" r:id="rId153"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H159" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H161" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H162" r:id="rId156"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId155"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId157"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda local de la mañana 2026-10-15 (Mac): 6 precios nuevos, 5 chats nuevos, primera cuenta de demanda, SpeedX entregado en Miami
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H189" headerRowCount="1">
-  <autoFilter ref="A1:H189"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H196" headerRowCount="1">
+  <autoFilter ref="A1:H196"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -785,12 +785,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>SSD NVMe 2TB</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -799,17 +799,17 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>142.24</v>
+        <v>209.99</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>120</v>
+        <v>175</v>
       </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="8" t="n">
-        <v>2860</v>
+        <v>4060</v>
       </c>
       <c r="I5" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -820,7 +820,7 @@
         <v/>
       </c>
       <c r="K5" s="8" t="n">
-        <v>350</v>
+        <v>80</v>
       </c>
       <c r="L5" s="11">
         <f>IF(D5="","",MIN(MAX(Supuestos!$B$5,CEILING((K5*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D5*Supuestos!$B$9))</f>
@@ -850,12 +850,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 2TB</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -864,17 +864,17 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>209.99</v>
+        <v>142.24</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>175</v>
+        <v>120</v>
       </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="8" t="n">
-        <v>4060</v>
+        <v>2800</v>
       </c>
       <c r="I6" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -885,7 +885,7 @@
         <v/>
       </c>
       <c r="K6" s="8" t="n">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="L6" s="11">
         <f>IF(D6="","",MIN(MAX(Supuestos!$B$5,CEILING((K6*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D6*Supuestos!$B$9))</f>
@@ -980,7 +980,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-12400F</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -994,17 +994,19 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>150</v>
+        <v>320</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>114.99</v>
-      </c>
-      <c r="G8" s="2" t="n"/>
+        <v>279.99</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>4800</v>
+      </c>
       <c r="H8" s="8" t="n">
-        <v>2460</v>
+        <v>4760</v>
       </c>
       <c r="I8" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1015,7 +1017,7 @@
         <v/>
       </c>
       <c r="K8" s="8" t="n">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="L8" s="11">
         <f>IF(D8="","",MIN(MAX(Supuestos!$B$5,CEILING((K8*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D8*Supuestos!$B$9))</f>
@@ -1045,7 +1047,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core i5-14400F</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1059,19 +1061,17 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>320</v>
+        <v>164.49</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>279.99</v>
-      </c>
-      <c r="G9" s="8" t="n">
-        <v>4800</v>
-      </c>
+        <v>134.99</v>
+      </c>
+      <c r="G9" s="2" t="n"/>
       <c r="H9" s="8" t="n">
-        <v>4760</v>
+        <v>2460</v>
       </c>
       <c r="I9" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1082,7 +1082,7 @@
         <v/>
       </c>
       <c r="K9" s="8" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="L9" s="11">
         <f>IF(D9="","",MIN(MAX(Supuestos!$B$5,CEILING((K9*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D9*Supuestos!$B$9))</f>
@@ -1112,7 +1112,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-14400F</t>
+          <t>Intel Core i5-12400F</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1126,17 +1126,17 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>164.49</v>
+        <v>150</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>134.99</v>
+        <v>114.99</v>
       </c>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="8" t="n">
-        <v>2460</v>
+        <v>2260</v>
       </c>
       <c r="I10" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -2056,7 +2056,9 @@
         <v>279.99</v>
       </c>
       <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="8" t="n">
+        <v>5890</v>
+      </c>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2164,7 +2166,9 @@
         <v>120</v>
       </c>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="8" t="n">
+        <v>2800</v>
+      </c>
       <c r="H7" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A7,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A7,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2329,7 +2333,9 @@
         <v>134.99</v>
       </c>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
+      <c r="G10" s="8" t="n">
+        <v>2750</v>
+      </c>
       <c r="H10" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2437,7 +2443,9 @@
         <v>114.99</v>
       </c>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="8" t="n">
+        <v>2260</v>
+      </c>
       <c r="H12" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A12,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A12,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -5905,7 +5913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13079,6 +13087,244 @@
         </is>
       </c>
       <c r="H189" s="2" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D190" s="5" t="inlineStr">
+        <is>
+          <t>SMART CUBE (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E190" s="11" t="n">
+        <v>5890</v>
+      </c>
+      <c r="F190" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G190" s="5" t="inlineStr">
+        <is>
+          <t>nuevo sellado, facturado; llevando 2 rebajan Bs 50 c/u (Bs 5.840)</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>SMART CUBE (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E191" s="11" t="n">
+        <v>3080</v>
+      </c>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>nuevo sellado; llevando 2 rebajan Bs 50 c/u (Bs 3.030)</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR5 16GB 6000 (Apacer NOX)</t>
+        </is>
+      </c>
+      <c r="D192" s="5" t="inlineStr">
+        <is>
+          <t>SMART CUBE (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E192" s="11" t="n">
+        <v>3650</v>
+      </c>
+      <c r="F192" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G192" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (Apacer NOX DDR5 16GB 6000: otra marca y capacidad; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR5 16GB</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>PC Factor (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E193" s="11" t="n">
+        <v>3792</v>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (USD 320 c/u a Bs 11,85; marca y velocidad por confirmar; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="D194" s="5" t="inlineStr">
+        <is>
+          <t>OverCity (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E194" s="11" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F194" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G194" s="5" t="inlineStr">
+        <is>
+          <t>OEM</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-12400F</t>
+        </is>
+      </c>
+      <c r="D195" s="5" t="inlineStr">
+        <is>
+          <t>T&amp;T Todo en Tecnología (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E195" s="11" t="n">
+        <v>2260</v>
+      </c>
+      <c r="F195" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G195" s="5" t="inlineStr">
+        <is>
+          <t>OEM con cooler Intel; Bs 20 menos c/u llevando 2</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B196" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D196" s="5" t="inlineStr">
+        <is>
+          <t>T&amp;T Todo en Tecnología (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E196" s="11" t="n">
+        <v>2750</v>
+      </c>
+      <c r="F196" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G196" s="5" t="inlineStr">
+        <is>
+          <t>OEM con cooler Intel; Bs 20 menos c/u llevando 2</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Repaso de la tarde 2026-10-15 (Mac, la PC no corrió): 4 respuestas de WhatsApp (Geek Store 7700X Bs 3.480), Soft Computers consultado, calles de Baton Rouge, Shreveport y Memphis para el mapa
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H196" headerRowCount="1">
-  <autoFilter ref="A1:H196"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H198" headerRowCount="1">
+  <autoFilter ref="A1:H198"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -5913,7 +5913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H196"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13325,6 +13325,74 @@
         </is>
       </c>
       <c r="H196" s="2" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7700X</t>
+        </is>
+      </c>
+      <c r="D197" s="5" t="inlineStr">
+        <is>
+          <t>Geek Store Bolivia (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E197" s="11" t="n">
+        <v>3480</v>
+      </c>
+      <c r="F197" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G197" s="5" t="inlineStr">
+        <is>
+          <t>sin confirmar si es sellado (se preguntó)</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B198" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>Kingston Fury DDR5 16GB (1 módulo)</t>
+        </is>
+      </c>
+      <c r="D198" s="5" t="inlineStr">
+        <is>
+          <t>Geek Store Bolivia (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E198" s="11" t="n">
+        <v>2900</v>
+      </c>
+      <c r="F198" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G198" s="5" t="inlineStr">
+        <is>
+          <t>otra marca; velocidad por confirmar (no es la Corsair 32GB 2x16)</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Catálogo de Shopping PC bajado y leído: lista mayorista en USD (100+ productos); SSD Kingston NV3 1TB Bs 1.754 cuenta, i5-14400 BOX y DDR4 16GB como referencia; Shopping PC pasa al grupo C; tarea 2026-10-16-1 hecha
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H198" headerRowCount="1">
-  <autoFilter ref="A1:H198"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H202" headerRowCount="1">
+  <autoFilter ref="A1:H202"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -1268,7 +1268,7 @@
         <v>1800</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>1860</v>
+        <v>1754</v>
       </c>
       <c r="I12" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1946,7 +1946,9 @@
         <v>80</v>
       </c>
       <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="8" t="n">
+        <v>1754</v>
+      </c>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -5913,7 +5915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13393,6 +13395,142 @@
         </is>
       </c>
       <c r="H198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B199" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D199" s="5" t="inlineStr">
+        <is>
+          <t>Shopping PC (catálogo PDF)</t>
+        </is>
+      </c>
+      <c r="E199" s="11" t="n">
+        <v>1754</v>
+      </c>
+      <c r="F199" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G199" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (Kingston NV3 1TB; lista mayorista USD 148 del 12/10, sin factura; 146 en stock)</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B200" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D200" s="5" t="inlineStr">
+        <is>
+          <t>Shopping PC (catálogo PDF)</t>
+        </is>
+      </c>
+      <c r="E200" s="11" t="n">
+        <v>2785</v>
+      </c>
+      <c r="F200" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G200" s="5" t="inlineStr">
+        <is>
+          <t>nuevo en caja (es el i5-14400 BOX con gráficos, no el F; lista mayorista USD 235, sin factura; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B201" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C201" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D201" s="5" t="inlineStr">
+        <is>
+          <t>Shopping PC (catálogo PDF)</t>
+        </is>
+      </c>
+      <c r="E201" s="11" t="n">
+        <v>1778</v>
+      </c>
+      <c r="F201" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G201" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (Kingston 16GB DDR4 3200, un módulo, no kit 2x8; lista mayorista USD 150; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="15" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B202" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C202" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D202" s="5" t="inlineStr">
+        <is>
+          <t>Shopping PC (catálogo PDF)</t>
+        </is>
+      </c>
+      <c r="E202" s="11" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F202" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G202" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (Musking Redline 16GB DDR4 3200, un módulo, no kit 2x8; lista mayorista USD 135; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ronda Mac 16/10: 4 respuestas de WhatsApp (14400F Bs 2.500 en Soft Computers), 1 chat nuevo (Punto Tecnológico), precios web de Cyrex, cuenta de demanda en Marketplace, USPS de prueba salió de Memphis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H228" headerRowCount="1">
-  <autoFilter ref="A1:H228"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H233" headerRowCount="1">
+  <autoFilter ref="A1:H233"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -1070,7 +1070,7 @@
         <v>80</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>1800</v>
+        <v>1730</v>
       </c>
       <c r="H9" s="8" t="n">
         <v>1754</v>
@@ -1114,7 +1114,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-14400F</t>
+          <t>Intel Core i5-12400F</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1128,17 +1128,17 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>164.49</v>
+        <v>150</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>139.99</v>
+        <v>120.99</v>
       </c>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="8" t="n">
-        <v>2460</v>
+        <v>2260</v>
       </c>
       <c r="I10" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1179,7 +1179,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-12400F</t>
+          <t>Intel Core i5-14400F</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1193,17 +1193,17 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>150</v>
+        <v>164.49</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>120.99</v>
+        <v>139.99</v>
       </c>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="8" t="n">
-        <v>2260</v>
+        <v>2384</v>
       </c>
       <c r="I11" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1945,7 +1945,9 @@
       <c r="E3" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="8" t="n">
+        <v>1730</v>
+      </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
@@ -2056,7 +2058,9 @@
         <v>279.99</v>
       </c>
       <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="8" t="n">
+        <v>5664</v>
+      </c>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2329,7 +2333,9 @@
         <v>139.99</v>
       </c>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
+      <c r="G10" s="8" t="n">
+        <v>2384</v>
+      </c>
       <c r="H10" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A10,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -6721,7 +6727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H228"/>
+  <dimension ref="A1:H233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15325,6 +15331,192 @@
         </is>
       </c>
       <c r="H228" s="2" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="15" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B229" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C229" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D229" s="5" t="inlineStr">
+        <is>
+          <t>Soft Computers (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E229" s="11" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F229" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G229" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM; mismo precio por unidad llevando 2</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="15" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B230" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C230" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D230" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba</t>
+        </is>
+      </c>
+      <c r="E230" s="11" t="n">
+        <v>1730</v>
+      </c>
+      <c r="F230" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G230" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (M.2 1TB, marca no indicada; publicado hace 2 días)</t>
+        </is>
+      </c>
+      <c r="H230" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="15" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B231" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C231" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D231" s="5" t="inlineStr">
+        <is>
+          <t>Cyrex Store (web)</t>
+        </is>
+      </c>
+      <c r="E231" s="11" t="n">
+        <v>2384</v>
+      </c>
+      <c r="F231" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G231" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (web: USD 202 a la tasa de la tienda, 11,80; hay otra publicación del mismo a USD 215)</t>
+        </is>
+      </c>
+      <c r="H231" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="15" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B232" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C232" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D232" s="5" t="inlineStr">
+        <is>
+          <t>Cyrex Store (web)</t>
+        </is>
+      </c>
+      <c r="E232" s="11" t="n">
+        <v>5664</v>
+      </c>
+      <c r="F232" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G232" s="5" t="inlineStr">
+        <is>
+          <t>nuevo BOX (web: USD 480 a 11,80)</t>
+        </is>
+      </c>
+      <c r="H232" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="15" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B233" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C233" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-13400</t>
+        </is>
+      </c>
+      <c r="D233" s="5" t="inlineStr">
+        <is>
+          <t>Cyrex Store (web)</t>
+        </is>
+      </c>
+      <c r="E233" s="11" t="n">
+        <v>2218</v>
+      </c>
+      <c r="F233" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G233" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (web: es el i5-13400F, sin gráficos; USD 188 a 11,80; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H233" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -15536,10 +15728,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H211" r:id="rId206"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H213" r:id="rId207"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H214" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H230" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H231" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H232" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H233" r:id="rId212"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId209"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId213"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda Mac 17/10: Pedidos (USPS de prueba llega el lunes 19/10), Marketplace (SSD 1TB nuevo a Bs 1.230), demanda, regenerado y oficina publicada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H259" headerRowCount="1">
-  <autoFilter ref="A1:H259"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H265" headerRowCount="1">
+  <autoFilter ref="A1:H265"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -1242,12 +1242,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>RAM</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1256,20 +1256,18 @@
         </is>
       </c>
       <c r="D12" s="7" t="n">
-        <v>128.99</v>
+        <v>429.97</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>98.59</v>
+        <v>375</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>1730</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>1754</v>
-      </c>
+        <v>4500</v>
+      </c>
+      <c r="H12" s="2" t="n"/>
       <c r="I12" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1279,7 +1277,7 @@
         <v/>
       </c>
       <c r="K12" s="8" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="L12" s="11">
         <f>IF(D12="","",MIN(MAX(Supuestos!$B$5,CEILING((K12*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D12*Supuestos!$B$9))</f>
@@ -1309,12 +1307,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+          <t>Ryzen 9 9950X</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>RAM</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1323,18 +1321,18 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>429.97</v>
+        <v>549.99</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>375</v>
-      </c>
-      <c r="G13" s="8" t="n">
-        <v>4500</v>
-      </c>
-      <c r="H13" s="2" t="n"/>
+        <v>454.99</v>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="8" t="n">
+        <v>5580</v>
+      </c>
       <c r="I13" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1344,7 +1342,7 @@
         <v/>
       </c>
       <c r="K13" s="8" t="n">
-        <v>150</v>
+        <v>350</v>
       </c>
       <c r="L13" s="11">
         <f>IF(D13="","",MIN(MAX(Supuestos!$B$5,CEILING((K13*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D13*Supuestos!$B$9))</f>
@@ -1374,12 +1372,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 9 9950X</t>
+          <t>SSD NVMe 1TB</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1388,17 +1386,19 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>549.99</v>
+        <v>128.99</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>454.99</v>
-      </c>
-      <c r="G14" s="2" t="n"/>
+        <v>98.59</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>1230</v>
+      </c>
       <c r="H14" s="8" t="n">
-        <v>5580</v>
+        <v>1754</v>
       </c>
       <c r="I14" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1409,7 +1409,7 @@
         <v/>
       </c>
       <c r="K14" s="8" t="n">
-        <v>350</v>
+        <v>80</v>
       </c>
       <c r="L14" s="11">
         <f>IF(D14="","",MIN(MAX(Supuestos!$B$5,CEILING((K14*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D14*Supuestos!$B$9))</f>
@@ -1945,7 +1945,9 @@
       <c r="E3" s="7" t="n">
         <v>98.59</v>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="8" t="n">
+        <v>1230</v>
+      </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
@@ -2934,7 +2936,9 @@
         <v>120</v>
       </c>
       <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
+      <c r="G21" s="8" t="n">
+        <v>2850</v>
+      </c>
       <c r="H21" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A21,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A21,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -7533,7 +7537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H259"/>
+  <dimension ref="A1:H265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17307,6 +17311,222 @@
         </is>
       </c>
       <c r="H259" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="15" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B260" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C260" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="D260" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E260" s="11" t="n">
+        <v>2850</v>
+      </c>
+      <c r="F260" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G260" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM, garantía 6 meses (cotización por WhatsApp)</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="15" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B261" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C261" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D261" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E261" s="11" t="n">
+        <v>5960</v>
+      </c>
+      <c r="F261" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G261" s="5" t="inlineStr">
+        <is>
+          <t>otra marca (Nox Tuf 32GB 2x16, velocidad sin dato); solo referencia; no cuenta</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="15" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B262" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C262" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="D262" s="5" t="inlineStr">
+        <is>
+          <t>Gamer Store Cbba (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E262" s="11" t="n">
+        <v>2067</v>
+      </c>
+      <c r="F262" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G262" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (es el 7600X; USD 175 a 11,81; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="15" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B263" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C263" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D263" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E263" s="11" t="n">
+        <v>1230</v>
+      </c>
+      <c r="F263" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G263" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (antes Bs 1.730; marca sin dato)</t>
+        </is>
+      </c>
+      <c r="H263" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="15" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B264" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C264" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D264" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E264" s="11" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F264" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G264" s="5" t="inlineStr">
+        <is>
+          <t>sin dato de estado ni marca (recién publicado)</t>
+        </is>
+      </c>
+      <c r="H264" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="15" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B265" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C265" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D265" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E265" s="11" t="n">
+        <v>1850</v>
+      </c>
+      <c r="F265" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G265" s="5" t="inlineStr">
+        <is>
+          <t>Kingston NV3 1TB (estado sin dato)</t>
+        </is>
+      </c>
+      <c r="H265" s="6" t="inlineStr">
         <is>
           <t>ver</t>
         </is>
@@ -17552,10 +17772,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H257" r:id="rId236"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H258" r:id="rId237"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H259" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H263" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H264" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H265" r:id="rId241"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId239"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId242"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda Mac 19/10: pedidos, análisis, finanzas y oficina publicada
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H318" headerRowCount="1">
-  <autoFilter ref="A1:H318"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H324" headerRowCount="1">
+  <autoFilter ref="A1:H324"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -785,12 +785,12 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 2TB</t>
+          <t>Ryzen 5 7600</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -799,17 +799,17 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>209.99</v>
+        <v>140.26</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>154.99</v>
+        <v>120</v>
       </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="8" t="n">
-        <v>4060</v>
+        <v>2800</v>
       </c>
       <c r="I5" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -820,7 +820,7 @@
         <v/>
       </c>
       <c r="K5" s="8" t="n">
-        <v>80</v>
+        <v>350</v>
       </c>
       <c r="L5" s="11">
         <f>IF(D5="","",MIN(MAX(Supuestos!$B$5,CEILING((K5*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D5*Supuestos!$B$9))</f>
@@ -850,12 +850,12 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Intel Core Ultra 7 265K</t>
+          <t>SSD NVMe 2TB</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -864,17 +864,17 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>230</v>
+        <v>209.99</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>5.27</v>
+        <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>239.99</v>
+        <v>154.99</v>
       </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="8" t="n">
-        <v>3950</v>
+        <v>4060</v>
       </c>
       <c r="I6" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -885,7 +885,7 @@
         <v/>
       </c>
       <c r="K6" s="8" t="n">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="L6" s="11">
         <f>IF(D6="","",MIN(MAX(Supuestos!$B$5,CEILING((K6*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D6*Supuestos!$B$9))</f>
@@ -915,7 +915,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core Ultra 7 265K</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -929,19 +929,17 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>324.99</v>
+        <v>230</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0</v>
+        <v>5.27</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>285</v>
-      </c>
-      <c r="G7" s="8" t="n">
-        <v>4800</v>
-      </c>
+        <v>239.99</v>
+      </c>
+      <c r="G7" s="2" t="n"/>
       <c r="H7" s="8" t="n">
-        <v>4760</v>
+        <v>3950</v>
       </c>
       <c r="I7" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -952,7 +950,7 @@
         <v/>
       </c>
       <c r="K7" s="8" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="L7" s="11">
         <f>IF(D7="","",MIN(MAX(Supuestos!$B$5,CEILING((K7*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D7*Supuestos!$B$9))</f>
@@ -982,7 +980,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-12400F</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -996,17 +994,19 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>150</v>
+        <v>324.99</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>124.99</v>
-      </c>
-      <c r="G8" s="2" t="n"/>
+        <v>285</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>4800</v>
+      </c>
       <c r="H8" s="8" t="n">
-        <v>2260</v>
+        <v>4760</v>
       </c>
       <c r="I8" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1017,7 +1017,7 @@
         <v/>
       </c>
       <c r="K8" s="8" t="n">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="L8" s="11">
         <f>IF(D8="","",MIN(MAX(Supuestos!$B$5,CEILING((K8*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D8*Supuestos!$B$9))</f>
@@ -1047,12 +1047,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+          <t>Intel Core i5-12400F</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>RAM</t>
+          <t>CPU</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1061,18 +1061,18 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>419.99</v>
-      </c>
-      <c r="G9" s="8" t="n">
-        <v>6200</v>
-      </c>
-      <c r="H9" s="2" t="n"/>
+        <v>124.99</v>
+      </c>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="8" t="n">
+        <v>2260</v>
+      </c>
       <c r="I9" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1082,7 +1082,7 @@
         <v/>
       </c>
       <c r="K9" s="8" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="L9" s="11">
         <f>IF(D9="","",MIN(MAX(Supuestos!$B$5,CEILING((K9*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D9*Supuestos!$B$9))</f>
@@ -1177,12 +1177,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 5 7600</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>RAM</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1191,18 +1191,18 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>213.95</v>
+        <v>450</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>120</v>
-      </c>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="8" t="n">
-        <v>2800</v>
-      </c>
+        <v>419.99</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>5800</v>
+      </c>
+      <c r="H11" s="2" t="n"/>
       <c r="I11" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1212,7 +1212,7 @@
         <v/>
       </c>
       <c r="K11" s="8" t="n">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="L11" s="11">
         <f>IF(D11="","",MIN(MAX(Supuestos!$B$5,CEILING((K11*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D11*Supuestos!$B$9))</f>
@@ -1945,7 +1945,9 @@
       <c r="E3" s="7" t="n">
         <v>95</v>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="8" t="n">
+        <v>2050</v>
+      </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
@@ -2158,7 +2160,7 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>213.95</v>
+        <v>140.26</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>120</v>
@@ -2546,7 +2548,9 @@
       <c r="E14" s="7" t="n">
         <v>419.99</v>
       </c>
-      <c r="F14" s="2" t="n"/>
+      <c r="F14" s="8" t="n">
+        <v>5800</v>
+      </c>
       <c r="G14" s="2" t="n"/>
       <c r="H14" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A14,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A14,Dólar!$A:$A,0))),"")</f>
@@ -9149,7 +9153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H318"/>
+  <dimension ref="A1:H324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17204,7 +17208,7 @@
         </is>
       </c>
       <c r="E212" s="11" t="n">
-        <v>213.95</v>
+        <v>140.26</v>
       </c>
       <c r="F212" s="5" t="inlineStr">
         <is>
@@ -17213,7 +17217,7 @@
       </c>
       <c r="G212" s="5" t="inlineStr">
         <is>
-          <t>eBay API; vendedor bra_dewaa 99.8%; AMD Ryzen 5 7600 6-Core 12-Thread Unlocked Desktop Processor</t>
+          <t>eBay Chrome 19/10 10:40: anuncio activo de Silaxon_Electronics 99.6% (20.397 valoraciones), Nuevo, envío gratis, ubicado en NJ, verificado en la página y en búsqueda; la API traía 213.95 (bra_dewaa 99.8%) y el 140.26 apareció después (anuncio nuevo)</t>
         </is>
       </c>
       <c r="H212" s="6" t="inlineStr">
@@ -21153,6 +21157,234 @@
         </is>
       </c>
       <c r="H318" s="2" t="n"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B319" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C319" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 5600</t>
+        </is>
+      </c>
+      <c r="D319" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E319" s="11" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F319" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G319" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: otro modelo (es 5600X, solo procesador, recién publicado)</t>
+        </is>
+      </c>
+      <c r="H319" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B320" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C320" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-13400</t>
+        </is>
+      </c>
+      <c r="D320" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E320" s="11" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F320" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G320" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: otro modelo (i5-13400F, precio fijo)</t>
+        </is>
+      </c>
+      <c r="H320" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B321" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C321" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-14400F</t>
+        </is>
+      </c>
+      <c r="D321" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E321" s="11" t="n">
+        <v>2600</v>
+      </c>
+      <c r="F321" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G321" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: otro modelo (i5-14400 sin F)</t>
+        </is>
+      </c>
+      <c r="H321" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B322" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C322" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D322" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E322" s="11" t="n">
+        <v>5800</v>
+      </c>
+      <c r="F322" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G322" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB 2x16 6000 MHz (estado sin dato)</t>
+        </is>
+      </c>
+      <c r="H322" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B323" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C323" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D323" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E323" s="11" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F323" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G323" s="5" t="inlineStr">
+        <is>
+          <t>Lexar NM790 1TB con disipador (estado sin dato)</t>
+        </is>
+      </c>
+      <c r="H323" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B324" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C324" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D324" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E324" s="11" t="n">
+        <v>2050</v>
+      </c>
+      <c r="F324" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G324" s="5" t="inlineStr">
+        <is>
+          <t>WD Green SN3000 1TB (estado sin dato)</t>
+        </is>
+      </c>
+      <c r="H324" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -21449,10 +21681,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H315" r:id="rId291"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H316" r:id="rId292"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H317" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H319" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H320" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H321" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H322" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H323" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H324" r:id="rId299"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId294"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId300"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda PC tarde 19/10: WhatsApp, Marketplace, Pedidos, Analista (mediana), Finanzas, oficina v69, Gerente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H324" headerRowCount="1">
-  <autoFilter ref="A1:H324"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H326" headerRowCount="1">
+  <autoFilter ref="A1:H326"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2166,7 +2166,9 @@
         <v>120</v>
       </c>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="8" t="n">
+        <v>2800</v>
+      </c>
       <c r="H7" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A7,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A7,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2494,7 +2496,9 @@
         <v>239.99</v>
       </c>
       <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
+      <c r="G13" s="8" t="n">
+        <v>4100</v>
+      </c>
       <c r="H13" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A13,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A13,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -9153,7 +9157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H324"/>
+  <dimension ref="A1:H326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21385,6 +21389,74 @@
           <t>ver</t>
         </is>
       </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B325" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C325" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="D325" s="5" t="inlineStr">
+        <is>
+          <t>OverCity (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E325" s="11" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F325" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G325" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM (reconfirmado 16:09)</t>
+        </is>
+      </c>
+      <c r="H325" s="2" t="n"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="15" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B326" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C326" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="D326" s="5" t="inlineStr">
+        <is>
+          <t>OverCity (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E326" s="11" t="n">
+        <v>4100</v>
+      </c>
+      <c r="F326" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G326" s="5" t="inlineStr">
+        <is>
+          <t>nuevo OEM</t>
+        </is>
+      </c>
+      <c r="H326" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ronda Mac 20/10: análisis, finanzas, reportes y oficina v70
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H351" headerRowCount="1">
-  <autoFilter ref="A1:H351"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H355" headerRowCount="1">
+  <autoFilter ref="A1:H355"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2055,7 +2055,9 @@
       <c r="E5" s="7" t="n">
         <v>289.99</v>
       </c>
-      <c r="F5" s="2" t="n"/>
+      <c r="F5" s="8" t="n">
+        <v>5390</v>
+      </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
@@ -2273,7 +2275,9 @@
       <c r="E9" s="7" t="n">
         <v>69.95</v>
       </c>
-      <c r="F9" s="2" t="n"/>
+      <c r="F9" s="8" t="n">
+        <v>1400</v>
+      </c>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A9,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A9,Dólar!$A:$A,0))),"")</f>
@@ -9961,7 +9965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H351"/>
+  <dimension ref="A1:H355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23211,6 +23215,150 @@
         </is>
       </c>
       <c r="H351" s="2" t="n"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B352" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C352" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D352" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E352" s="11" t="n">
+        <v>5190</v>
+      </c>
+      <c r="F352" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G352" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: anuncio viejo (nuevo; publicado hace 13 semanas)</t>
+        </is>
+      </c>
+      <c r="H352" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B353" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C353" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D353" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E353" s="11" t="n">
+        <v>5390</v>
+      </c>
+      <c r="F353" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G353" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (anuncio 'El mejor para Gaming'; disponible)</t>
+        </is>
+      </c>
+      <c r="H353" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B354" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C354" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="D354" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace La Paz (particular)</t>
+        </is>
+      </c>
+      <c r="E354" s="11" t="n">
+        <v>3950</v>
+      </c>
+      <c r="F354" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G354" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: otra ciudad (La Paz; nuevo)</t>
+        </is>
+      </c>
+      <c r="H354" s="2" t="n"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="15" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B355" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C355" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D355" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E355" s="11" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F355" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G355" s="5" t="inlineStr">
+        <is>
+          <t>2x8 = 16GB (marca y frecuencia sin dato; antes Bs 1.600; vuelve a aparecer)</t>
+        </is>
+      </c>
+      <c r="H355" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -23538,10 +23686,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H347" r:id="rId322"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H348" r:id="rId323"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H349" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H352" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H353" r:id="rId326"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId325"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId327"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda Mac 21/10: oficina v73, reportes y métricas
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H396" headerRowCount="1">
-  <autoFilter ref="A1:H396"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H402" headerRowCount="1">
+  <autoFilter ref="A1:H402"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -1071,7 +1071,9 @@
       <c r="F9" s="7" t="n">
         <v>124</v>
       </c>
-      <c r="G9" s="2" t="n"/>
+      <c r="G9" s="8" t="n">
+        <v>2350</v>
+      </c>
       <c r="H9" s="8" t="n">
         <v>2260</v>
       </c>
@@ -2077,7 +2079,9 @@
       <c r="E3" s="7" t="n">
         <v>90</v>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="8" t="n">
+        <v>1700</v>
+      </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
@@ -2187,7 +2191,9 @@
       <c r="E5" s="7" t="n">
         <v>289.99</v>
       </c>
-      <c r="F5" s="2" t="n"/>
+      <c r="F5" s="8" t="n">
+        <v>4860</v>
+      </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
@@ -2243,7 +2249,9 @@
         <v>189.99</v>
       </c>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="8" t="n">
+        <v>3480</v>
+      </c>
       <c r="H6" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A6,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A6,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -2676,7 +2684,9 @@
       <c r="E14" s="7" t="n">
         <v>124</v>
       </c>
-      <c r="F14" s="2" t="n"/>
+      <c r="F14" s="8" t="n">
+        <v>2350</v>
+      </c>
       <c r="G14" s="2" t="n"/>
       <c r="H14" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A14,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A14,Dólar!$A:$A,0))),"")</f>
@@ -2786,7 +2796,9 @@
       <c r="E16" s="7" t="n">
         <v>399.99</v>
       </c>
-      <c r="F16" s="2" t="n"/>
+      <c r="F16" s="8" t="n">
+        <v>6200</v>
+      </c>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A16,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A16,Dólar!$A:$A,0))),"")</f>
@@ -11120,7 +11132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H396"/>
+  <dimension ref="A1:H402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26072,6 +26084,210 @@
           <t>ver</t>
         </is>
       </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B397" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C397" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7700X</t>
+        </is>
+      </c>
+      <c r="D397" s="5" t="inlineStr">
+        <is>
+          <t>Geek Store Bolivia (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E397" s="11" t="n">
+        <v>3480</v>
+      </c>
+      <c r="F397" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G397" s="5" t="inlineStr">
+        <is>
+          <t>nuevo sellado (caja)</t>
+        </is>
+      </c>
+      <c r="H397" s="2" t="n"/>
+    </row>
+    <row r="398">
+      <c r="A398" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B398" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C398" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core i5-12400F</t>
+        </is>
+      </c>
+      <c r="D398" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E398" s="11" t="n">
+        <v>2350</v>
+      </c>
+      <c r="F398" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G398" s="5" t="inlineStr">
+        <is>
+          <t>OEM (anuncio "Procesador CPU i5 12400f OEM"; estado sin dato)</t>
+        </is>
+      </c>
+      <c r="H398" s="2" t="n"/>
+    </row>
+    <row r="399">
+      <c r="A399" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B399" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C399" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 6000</t>
+        </is>
+      </c>
+      <c r="D399" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E399" s="11" t="n">
+        <v>6200</v>
+      </c>
+      <c r="F399" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G399" s="5" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance RGB RS 2x16 6000 MHz ("última unidad"; estado sin dato)</t>
+        </is>
+      </c>
+      <c r="H399" s="2" t="n"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B400" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C400" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D400" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (tienda sin confirmar)</t>
+        </is>
+      </c>
+      <c r="E400" s="11" t="n">
+        <v>4860</v>
+      </c>
+      <c r="F400" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G400" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (anuncio multi-modelo "9800X3D, 7800X3D, 8700G"; precio desde)</t>
+        </is>
+      </c>
+      <c r="H400" s="2" t="n"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B401" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C401" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D401" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E401" s="11" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F401" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G401" s="5" t="inlineStr">
+        <is>
+          <t>Kingston NV2 NVMe 1TB (estado sin dato; recién publicado)</t>
+        </is>
+      </c>
+      <c r="H401" s="2" t="n"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B402" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C402" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D402" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E402" s="11" t="n">
+        <v>3050</v>
+      </c>
+      <c r="F402" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G402" s="5" t="inlineStr">
+        <is>
+          <t>Samsung 9100 PRO 1TB PCIe 5.0 (gama alta; estado sin dato)</t>
+        </is>
+      </c>
+      <c r="H402" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ronda PC tarde 21/10: WhatsApp, Marketplace, Pedidos, Analista, Finanzas, oficina v74 y aviso del Gerente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H402" headerRowCount="1">
-  <autoFilter ref="A1:H402"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H404" headerRowCount="1">
+  <autoFilter ref="A1:H404"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2194,7 +2194,9 @@
       <c r="F5" s="8" t="n">
         <v>4860</v>
       </c>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="8" t="n">
+        <v>6193</v>
+      </c>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -11132,7 +11134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H402"/>
+  <dimension ref="A1:H404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26288,6 +26290,74 @@
         </is>
       </c>
       <c r="H402" s="2" t="n"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B403" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C403" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D403" s="5" t="inlineStr">
+        <is>
+          <t>ADN Gamer Store (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E403" s="11" t="n">
+        <v>6193</v>
+      </c>
+      <c r="F403" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G403" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (estado y garantía sin confirmar; se preguntó)</t>
+        </is>
+      </c>
+      <c r="H403" s="2" t="n"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="15" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B404" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C404" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="D404" s="5" t="inlineStr">
+        <is>
+          <t>ADN Gamer Store (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E404" s="11" t="n">
+        <v>2918</v>
+      </c>
+      <c r="F404" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G404" s="5" t="inlineStr">
+        <is>
+          <t>nuevo (es el 7600X, no el 7600; USD 245 × 11,91; solo referencia; no cuenta)</t>
+        </is>
+      </c>
+      <c r="H404" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
PC cubre la ronda de la mañana de la Mac 22/10: WhatsApp, Instagram/Facebook, Marketplace, pedidos, análisis, finanzas, oficina v76 y aviso del Gerente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H433" headerRowCount="1">
-  <autoFilter ref="A1:H433"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H438" headerRowCount="1">
+  <autoFilter ref="A1:H438"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -850,7 +850,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7700X</t>
+          <t>Intel Core Ultra 7 265K</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -864,19 +864,17 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>212</v>
+        <v>243.6</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>189.99</v>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>4000</v>
-      </c>
+        <v>230</v>
+      </c>
+      <c r="G6" s="2" t="n"/>
       <c r="H6" s="8" t="n">
-        <v>3480</v>
+        <v>3950</v>
       </c>
       <c r="I6" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -887,7 +885,7 @@
         <v/>
       </c>
       <c r="K6" s="8" t="n">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="L6" s="11">
         <f>IF(D6="","",MIN(MAX(Supuestos!$B$5,CEILING((K6*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D6*Supuestos!$B$9))</f>
@@ -917,7 +915,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Intel Core Ultra 7 265K</t>
+          <t>Ryzen 7 7800X3D</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -931,17 +929,19 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>243.6</v>
+        <v>329</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>230</v>
-      </c>
-      <c r="G7" s="2" t="n"/>
+        <v>274.99</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>4800</v>
+      </c>
       <c r="H7" s="8" t="n">
-        <v>3950</v>
+        <v>4760</v>
       </c>
       <c r="I7" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -952,7 +952,7 @@
         <v/>
       </c>
       <c r="K7" s="8" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="L7" s="11">
         <f>IF(D7="","",MIN(MAX(Supuestos!$B$5,CEILING((K7*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D7*Supuestos!$B$9))</f>
@@ -982,7 +982,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Ryzen 7 7800X3D</t>
+          <t>Intel Core i5-12400F</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -996,19 +996,19 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>329</v>
+        <v>150</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>274.99</v>
+        <v>119.99</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>4800</v>
+        <v>2350</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>4760</v>
+        <v>2260</v>
       </c>
       <c r="I8" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1019,7 +1019,7 @@
         <v/>
       </c>
       <c r="K8" s="8" t="n">
-        <v>350</v>
+        <v>250</v>
       </c>
       <c r="L8" s="11">
         <f>IF(D8="","",MIN(MAX(Supuestos!$B$5,CEILING((K8*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D8*Supuestos!$B$9))</f>
@@ -1049,7 +1049,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Intel Core i5-12400F</t>
+          <t>Ryzen 7 7700X</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1063,19 +1063,19 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>150</v>
+        <v>212</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>119.99</v>
+        <v>189.99</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>2350</v>
+        <v>3100</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>2260</v>
+        <v>3480</v>
       </c>
       <c r="I9" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
@@ -1086,7 +1086,7 @@
         <v/>
       </c>
       <c r="K9" s="8" t="n">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="L9" s="11">
         <f>IF(D9="","",MIN(MAX(Supuestos!$B$5,CEILING((K9*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D9*Supuestos!$B$9))</f>
@@ -1596,7 +1596,7 @@
         <v>69.95</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>900</v>
+        <v>540</v>
       </c>
       <c r="H17" s="8" t="n">
         <v>2150</v>
@@ -2079,7 +2079,9 @@
       <c r="E3" s="7" t="n">
         <v>85</v>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="8" t="n">
+        <v>2050</v>
+      </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
@@ -2244,7 +2246,9 @@
       <c r="E6" s="7" t="n">
         <v>189.99</v>
       </c>
-      <c r="F6" s="2" t="n"/>
+      <c r="F6" s="8" t="n">
+        <v>3100</v>
+      </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A6,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A6,Dólar!$A:$A,0))),"")</f>
@@ -2517,7 +2521,9 @@
       <c r="E11" s="7" t="n">
         <v>69.95</v>
       </c>
-      <c r="F11" s="2" t="n"/>
+      <c r="F11" s="8" t="n">
+        <v>540</v>
+      </c>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A11,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A11,Dólar!$A:$A,0))),"")</f>
@@ -12050,7 +12056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H433"/>
+  <dimension ref="A1:H438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28376,6 +28382,196 @@
         </is>
       </c>
       <c r="H433" s="2" t="n"/>
+    </row>
+    <row r="434">
+      <c r="A434" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B434" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C434" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7700X</t>
+        </is>
+      </c>
+      <c r="D434" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E434" s="11" t="n">
+        <v>3100</v>
+      </c>
+      <c r="F434" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G434" s="5" t="inlineStr">
+        <is>
+          <t>estado sin dato (antes Bs 3.500 tachado; puede ser el mismo anuncio de Bs 3.000 de ayer con otro precio)</t>
+        </is>
+      </c>
+      <c r="H434" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B435" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C435" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D435" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E435" s="11" t="n">
+        <v>600</v>
+      </c>
+      <c r="F435" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G435" s="5" t="inlineStr">
+        <is>
+          <t>estado sin dato (2x8 16GB; recién publicado)</t>
+        </is>
+      </c>
+      <c r="H435" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B436" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C436" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D436" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E436" s="11" t="n">
+        <v>540</v>
+      </c>
+      <c r="F436" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G436" s="5" t="inlineStr">
+        <is>
+          <t>estado sin dato (Kingston Fury Beast RGB 16GB 3200; no queda claro si es 2x8 o un módulo)</t>
+        </is>
+      </c>
+      <c r="H436" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B437" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C437" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D437" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E437" s="11" t="n">
+        <v>2050</v>
+      </c>
+      <c r="F437" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G437" s="5" t="inlineStr">
+        <is>
+          <t>estado sin dato (WD Green SN3000 1TB)</t>
+        </is>
+      </c>
+      <c r="H437" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B438" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C438" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D438" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E438" s="11" t="n">
+        <v>2060</v>
+      </c>
+      <c r="F438" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G438" s="5" t="inlineStr">
+        <is>
+          <t>estado sin dato (WD Green SN3000 1TB)</t>
+        </is>
+      </c>
+      <c r="H438" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -28775,10 +28971,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H423" r:id="rId394"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H424" r:id="rId395"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H425" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H434" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H435" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H436" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H437" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H438" r:id="rId401"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId397"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId402"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
PC cubre la ronda de la mañana de la Mac 23/10: WhatsApp, Marketplace/Google Maps, pedidos, análisis, oficina v79 y aviso del Gerente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H468" headerRowCount="1">
-  <autoFilter ref="A1:H468"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H475" headerRowCount="1">
+  <autoFilter ref="A1:H475"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2517,7 +2517,9 @@
       <c r="E11" s="7" t="n">
         <v>64.98999999999999</v>
       </c>
-      <c r="F11" s="2" t="n"/>
+      <c r="F11" s="8" t="n">
+        <v>1600</v>
+      </c>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A11,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A11,Dólar!$A:$A,0))),"")</f>
@@ -12974,7 +12976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H468"/>
+  <dimension ref="A1:H475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30626,6 +30628,260 @@
         </is>
       </c>
       <c r="H468" s="2" t="n"/>
+    </row>
+    <row r="469">
+      <c r="A469" s="15" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B469" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C469" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="D469" s="5" t="inlineStr">
+        <is>
+          <t>TechMax Computers Cbba (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E469" s="11" t="n">
+        <v>4300</v>
+      </c>
+      <c r="F469" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G469" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: modelo sin confirmar (dijo 'Core Ultra 7'; se preguntó si es el 265K); sin garantía, traído de EEUU; estado 'perfecto estado'</t>
+        </is>
+      </c>
+      <c r="H469" s="2" t="n"/>
+    </row>
+    <row r="470">
+      <c r="A470" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B470" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C470" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 5600</t>
+        </is>
+      </c>
+      <c r="D470" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico · Supermall (web, vista en Google 23/10)</t>
+        </is>
+      </c>
+      <c r="E470" s="11" t="n">
+        <v>1710</v>
+      </c>
+      <c r="F470" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G470" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: agotado (referencia web; ya anotada el 12/10, la web sigue mostrando el mismo precio)</t>
+        </is>
+      </c>
+      <c r="H470" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B471" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C471" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 5700X3D</t>
+        </is>
+      </c>
+      <c r="D471" s="5" t="inlineStr">
+        <is>
+          <t>Facebook grupo TEAM PC's BOLIVIA (web, vista en Google 23/10)</t>
+        </is>
+      </c>
+      <c r="E471" s="11" t="n">
+        <v>3800</v>
+      </c>
+      <c r="F471" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G471" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: referencia vieja (comentario "de 3.800 Bs arriba" en el grupo TEAM PC's BOLIVIA; nuevo; sin ciudad ni anuncio)</t>
+        </is>
+      </c>
+      <c r="H471" s="2" t="n"/>
+    </row>
+    <row r="472">
+      <c r="A472" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B472" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C472" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7500F</t>
+        </is>
+      </c>
+      <c r="D472" s="5" t="inlineStr">
+        <is>
+          <t>Facebook grupo PC GAMERS BOLIVIA (web, vista en Google 23/10)</t>
+        </is>
+      </c>
+      <c r="E472" s="11" t="n">
+        <v>2050</v>
+      </c>
+      <c r="F472" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G472" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: referencia vieja (2 unidades nuevas "recién llegadas" en el grupo PC GAMERS BOLIVIA; sin ciudad)</t>
+        </is>
+      </c>
+      <c r="H472" s="2" t="n"/>
+    </row>
+    <row r="473">
+      <c r="A473" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B473" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C473" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D473" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E473" s="11" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F473" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G473" s="5" t="inlineStr">
+        <is>
+          <t>sin dato de estado (Corsair Vengeance Pro 2x8GB 3200 MHz)</t>
+        </is>
+      </c>
+      <c r="H473" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B474" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C474" s="5" t="inlineStr">
+        <is>
+          <t>RAM DDR4 16GB (2x8) 3200</t>
+        </is>
+      </c>
+      <c r="D474" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E474" s="11" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F474" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G474" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: velocidad sin dato (anuncio "Ram 2 x 8 = 16Gb"; estado sin dato; tachado Bs 1.600)</t>
+        </is>
+      </c>
+      <c r="H474" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B475" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C475" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 2TB</t>
+        </is>
+      </c>
+      <c r="D475" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E475" s="11" t="n">
+        <v>3350</v>
+      </c>
+      <c r="F475" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G475" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: tipo sin confirmar (anuncio "Sandisk SSD 2 TB recién llegadas"; tachado Bs 3.550; no dice si es NVMe o SATA)</t>
+        </is>
+      </c>
+      <c r="H475" s="6" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -31059,10 +31315,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H465" r:id="rId428"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H466" r:id="rId429"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H467" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H470" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H473" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H474" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H475" r:id="rId434"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId431"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId435"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ronda local de la tarde 23/10 (PC): WhatsApp, Marketplace, Pedidos, análisis, oficina v80 y aviso del Gerente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H475" headerRowCount="1">
-  <autoFilter ref="A1:H475"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H479" headerRowCount="1">
+  <autoFilter ref="A1:H479"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2245,7 +2245,9 @@
         <v>189.99</v>
       </c>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="8" t="n">
+        <v>3673.5</v>
+      </c>
       <c r="H6" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A6,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A6,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -12976,7 +12978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H475"/>
+  <dimension ref="A1:H479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30882,6 +30884,142 @@
           <t>ver</t>
         </is>
       </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B476" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C476" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7700X</t>
+        </is>
+      </c>
+      <c r="D476" s="5" t="inlineStr">
+        <is>
+          <t>Cyrex Store (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E476" s="11" t="n">
+        <v>3673.5</v>
+      </c>
+      <c r="F476" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G476" s="5" t="inlineStr">
+        <is>
+          <t>nuevo BOX (según foto de su chat; solo queda 1 unidad)</t>
+        </is>
+      </c>
+      <c r="H476" s="2" t="n"/>
+    </row>
+    <row r="477">
+      <c r="A477" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B477" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C477" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 5 7600</t>
+        </is>
+      </c>
+      <c r="D477" s="5" t="inlineStr">
+        <is>
+          <t>Nerd Tecnologias (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E477" s="11" t="n">
+        <v>2700</v>
+      </c>
+      <c r="F477" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G477" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: precio de segunda mano (lo consultó a un colega); estado y garantía sin confirmar</t>
+        </is>
+      </c>
+      <c r="H477" s="2" t="n"/>
+    </row>
+    <row r="478">
+      <c r="A478" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B478" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C478" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D478" s="5" t="inlineStr">
+        <is>
+          <t>Nerd Tecnologias (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E478" s="11" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F478" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G478" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: precio de segunda mano (colega); marca y tipo sin confirmar ("M2 de 1 tera")</t>
+        </is>
+      </c>
+      <c r="H478" s="2" t="n"/>
+    </row>
+    <row r="479">
+      <c r="A479" s="15" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B479" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C479" s="5" t="inlineStr">
+        <is>
+          <t>Intel Core Ultra 7 265K</t>
+        </is>
+      </c>
+      <c r="D479" s="5" t="inlineStr">
+        <is>
+          <t>TechMax Computers Cbba (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E479" s="11" t="n">
+        <v>4300</v>
+      </c>
+      <c r="F479" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G479" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: es el Core Ultra 7 270K (no el 265K); sin garantía, traído de EEUU</t>
+        </is>
+      </c>
+      <c r="H479" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ronda Mac 26/10: WhatsApp, Marketplace, demanda, Pedidos, Analista y Finanzas; quita el pedido cubre mac (la Mac sí hizo la ronda)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H568" headerRowCount="1">
-  <autoFilter ref="A1:H568"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H570" headerRowCount="1">
+  <autoFilter ref="A1:H570"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2079,7 +2079,9 @@
       <c r="E3" s="7" t="n">
         <v>85</v>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="8" t="n">
+        <v>1850</v>
+      </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
@@ -2189,7 +2191,9 @@
       <c r="E5" s="7" t="n">
         <v>269.99</v>
       </c>
-      <c r="F5" s="2" t="n"/>
+      <c r="F5" s="8" t="n">
+        <v>4800</v>
+      </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A5,Dólar!$A:$A,0))),"")</f>
@@ -15715,7 +15719,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>BCB oficial 11.88 (dolarbolivia.net 26/10 11:53 BOT</t>
+          <t>BCB oficial 11.88 (dolarbolivia.net 26/10 11:53 BOT, mismo dato que 25/10); paralelo dolarbolivia.net 26/10 (compra 11.97 / venta 11.96); usado = promedio del paralelo</t>
         </is>
       </c>
     </row>
@@ -15730,7 +15734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H568"/>
+  <dimension ref="A1:H570"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37154,6 +37158,74 @@
         </is>
       </c>
       <c r="H568" s="2" t="n"/>
+    </row>
+    <row r="569">
+      <c r="A569" s="15" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B569" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C569" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7800X3D</t>
+        </is>
+      </c>
+      <c r="D569" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E569" s="11" t="n">
+        <v>4800</v>
+      </c>
+      <c r="F569" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G569" s="5" t="inlineStr">
+        <is>
+          <t>nuevo sellado (anuncio "AMD Ryzen 7 7800X3D (Sellado)"; el vendedor dijo el 13/10 que acepta ofertas, no se oferta)</t>
+        </is>
+      </c>
+      <c r="H569" s="2" t="n"/>
+    </row>
+    <row r="570">
+      <c r="A570" s="15" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B570" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C570" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D570" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E570" s="11" t="n">
+        <v>1850</v>
+      </c>
+      <c r="F570" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G570" s="5" t="inlineStr">
+        <is>
+          <t>Kingston NV3 NVMe 1TB 6000MB/s (estado sin dato)</t>
+        </is>
+      </c>
+      <c r="H570" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ronda local de la tarde PC 26/10: WhatsApp, Instagram, pedidos, análisis, oficina v85 y aviso del Gerente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H570" headerRowCount="1">
-  <autoFilter ref="A1:H570"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H572" headerRowCount="1">
+  <autoFilter ref="A1:H572"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -2082,7 +2082,9 @@
       <c r="F3" s="8" t="n">
         <v>1850</v>
       </c>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="8" t="n">
+        <v>2000</v>
+      </c>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
         <v/>
@@ -15734,7 +15736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H570"/>
+  <dimension ref="A1:H572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37226,6 +37228,74 @@
         </is>
       </c>
       <c r="H570" s="2" t="n"/>
+    </row>
+    <row r="571">
+      <c r="A571" s="15" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B571" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C571" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D571" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E571" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F571" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G571" s="5" t="inlineStr">
+        <is>
+          <t>sin dato (modelo SN3000; falta confirmar NVMe, nuevo y garantía)</t>
+        </is>
+      </c>
+      <c r="H571" s="2" t="n"/>
+    </row>
+    <row r="572">
+      <c r="A572" s="15" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B572" s="5" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="C572" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 9700X</t>
+        </is>
+      </c>
+      <c r="D572" s="5" t="inlineStr">
+        <is>
+          <t>Punto Tecnológico (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E572" s="11" t="n">
+        <v>3680</v>
+      </c>
+      <c r="F572" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G572" s="5" t="inlineStr">
+        <is>
+          <t>no cuenta: no es producto de vigilar; OEM</t>
+        </is>
+      </c>
+      <c r="H572" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ronda Mac 28/10: 7700X entregados en la casilla, SSD 1TB con garantía, demanda y análisis con dólar 12,15
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H630" headerRowCount="1">
-  <autoFilter ref="A1:H630"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H633" headerRowCount="1">
+  <autoFilter ref="A1:H633"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -1376,12 +1376,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>SSD NVMe 1TB</t>
+          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>SSD</t>
+          <t>RAM</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1390,20 +1390,18 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>114.99</v>
+        <v>459</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>85</v>
+        <v>399.99</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>1230</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>1754</v>
-      </c>
+        <v>4500</v>
+      </c>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1413,7 +1411,7 @@
         <v/>
       </c>
       <c r="K14" s="8" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="L14" s="11">
         <f>IF(D14="","",MIN(MAX(Supuestos!$B$5,CEILING((K14*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D14*Supuestos!$B$9))</f>
@@ -1443,12 +1441,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Corsair Vengeance RGB DDR5 32GB (2x16) 5600</t>
+          <t>SSD NVMe 1TB</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>RAM</t>
+          <t>SSD</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1457,18 +1455,20 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>459</v>
+        <v>114.99</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>399.99</v>
+        <v>85</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>4500</v>
-      </c>
-      <c r="H15" s="2" t="n"/>
+        <v>1100</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>1754</v>
+      </c>
       <c r="I15" s="9">
         <f>INDEX(Dólar!$B:$B,MATCH(MAX(Dólar!$A:$A),Dólar!$A:$A,0))</f>
         <v/>
@@ -1478,7 +1478,7 @@
         <v/>
       </c>
       <c r="K15" s="8" t="n">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="L15" s="11">
         <f>IF(D15="","",MIN(MAX(Supuestos!$B$5,CEILING((K15*Supuestos!$B$3+Supuestos!$B$7)/1000,Supuestos!$B$6))*Supuestos!$B$4/Supuestos!$B$3,Supuestos!$B$8+D15*Supuestos!$B$9))</f>
@@ -2079,7 +2079,9 @@
       <c r="E3" s="7" t="n">
         <v>85</v>
       </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="F3" s="8" t="n">
+        <v>1100</v>
+      </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A3,Dólar!$A:$A,0))),"")</f>
@@ -2244,7 +2246,9 @@
       <c r="E6" s="7" t="n">
         <v>189.99</v>
       </c>
-      <c r="F6" s="2" t="n"/>
+      <c r="F6" s="8" t="n">
+        <v>4000</v>
+      </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="9">
         <f>IFERROR(IF(INDEX(Dólar!$B:$B,MATCH(A6,Dólar!$A:$A,0))="","",INDEX(Dólar!$B:$B,MATCH(A6,Dólar!$A:$A,0))),"")</f>
@@ -17568,7 +17572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H630"/>
+  <dimension ref="A1:H633"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41294,7 +41298,7 @@
       </c>
       <c r="G629" s="5" t="inlineStr">
         <is>
-          <t>sin dato (modelo SN3000; falta confirmar NVMe, nuevo y garantía)</t>
+          <t>nuevo, NVMe (modelo SN3000), garantía 6 meses (confirmado 28/10)</t>
         </is>
       </c>
       <c r="H629" s="2" t="n"/>
@@ -41332,6 +41336,108 @@
         </is>
       </c>
       <c r="H630" s="2" t="n"/>
+    </row>
+    <row r="631">
+      <c r="A631" s="15" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B631" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C631" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7 7700X</t>
+        </is>
+      </c>
+      <c r="D631" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E631" s="11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F631" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G631" s="5" t="inlineStr">
+        <is>
+          <t>nuevo sellado ("Ryzen 7 7700x Sellado"); Cochabamba</t>
+        </is>
+      </c>
+      <c r="H631" s="2" t="n"/>
+    </row>
+    <row r="632">
+      <c r="A632" s="15" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B632" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C632" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D632" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E632" s="11" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F632" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G632" s="5" t="inlineStr">
+        <is>
+          <t>Kingston NV2 NVMe PCIe 4.0 1TB (estado sin dato); Cochabamba</t>
+        </is>
+      </c>
+      <c r="H632" s="2" t="n"/>
+    </row>
+    <row r="633">
+      <c r="A633" s="15" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B633" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C633" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D633" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E633" s="11" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F633" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G633" s="5" t="inlineStr">
+        <is>
+          <t>"Disco duro m2 NVMe 1 tb" marca y estado sin dato; Cochabamba</t>
+        </is>
+      </c>
+      <c r="H633" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ronda PC tarde 28/10 (pedido del vigilante): WhatsApp, Marketplace, Pedidos, Analista, Finanzas, oficina v100, aviso del Gerente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importacion-cochabamba.xlsx
+++ b/importacion-cochabamba.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H633" headerRowCount="1">
-  <autoFilter ref="A1:H633"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Movimientos" displayName="Movimientos" ref="A1:H634" headerRowCount="1">
+  <autoFilter ref="A1:H634"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Fecha"/>
     <tableColumn id="2" name="Origen"/>
@@ -17572,7 +17572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H633"/>
+  <dimension ref="A1:H634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41438,6 +41438,40 @@
         </is>
       </c>
       <c r="H633" s="2" t="n"/>
+    </row>
+    <row r="634">
+      <c r="A634" s="15" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B634" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="C634" s="5" t="inlineStr">
+        <is>
+          <t>SSD NVMe 1TB</t>
+        </is>
+      </c>
+      <c r="D634" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace Cochabamba (particular)</t>
+        </is>
+      </c>
+      <c r="E634" s="11" t="n">
+        <v>1675</v>
+      </c>
+      <c r="F634" s="5" t="inlineStr">
+        <is>
+          <t>Bs</t>
+        </is>
+      </c>
+      <c r="G634" s="5" t="inlineStr">
+        <is>
+          <t>Kingston NV2 NVMe 1TB (estado sin dato; "SSD NV2 de 1TB"); Cochabamba</t>
+        </is>
+      </c>
+      <c r="H634" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>